<commit_message>
1) Agregue IACA a las correls de Arg 2) arregle imputacion ARG
</commit_message>
<xml_diff>
--- a/ARG/Covariables.xlsx
+++ b/ARG/Covariables.xlsx
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1378" uniqueCount="1066">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1380" uniqueCount="1068">
   <si>
     <t>Tea</t>
   </si>
@@ -3201,63 +3201,70 @@
     <t>Bono 10</t>
   </si>
   <si>
+    <t>ICC Michigan</t>
+  </si>
+  <si>
+    <t>NASDAQ</t>
+  </si>
+  <si>
+    <t>Bono 2</t>
+  </si>
+  <si>
+    <t>Gas Natural EEUU</t>
+  </si>
+  <si>
+    <t>Gas Natural Europa</t>
+  </si>
+  <si>
+    <t>Soja</t>
+  </si>
+  <si>
+    <t>Maiz</t>
+  </si>
+  <si>
+    <t>Sorgo</t>
+  </si>
+  <si>
+    <t>Trigo SRW</t>
+  </si>
+  <si>
+    <t>Trigo HRW</t>
+  </si>
+  <si>
+    <t>Carne</t>
+  </si>
+  <si>
+    <t>Pollo</t>
+  </si>
+  <si>
+    <t>FEFundsRate</t>
+  </si>
+  <si>
+    <t>Dow Jones</t>
+  </si>
+  <si>
+    <t>Petroleo Brent</t>
+  </si>
+  <si>
+    <t>Petroleo WTI</t>
+  </si>
+  <si>
     <t>ICC Di Tella</t>
   </si>
   <si>
-    <t>NASDAQ</t>
-  </si>
-  <si>
-    <t>Bono 2</t>
-  </si>
-  <si>
-    <t>Gas Natural EEUU</t>
-  </si>
-  <si>
-    <t>Gas Natural Europa</t>
-  </si>
-  <si>
-    <t>Soja</t>
-  </si>
-  <si>
-    <t>Maiz</t>
-  </si>
-  <si>
-    <t>Sorgo</t>
-  </si>
-  <si>
-    <t>Trigo SRW</t>
-  </si>
-  <si>
-    <t>Trigo HRW</t>
-  </si>
-  <si>
-    <t>Carne</t>
-  </si>
-  <si>
-    <t>Pollo</t>
-  </si>
-  <si>
-    <t>FEFundsRate</t>
-  </si>
-  <si>
-    <t>Dow Jones</t>
-  </si>
-  <si>
-    <t>Petroleo Brent</t>
-  </si>
-  <si>
-    <t>Petroleo WTI</t>
+    <t>IACA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="dd\-mm\-yy;@"/>
     <numFmt numFmtId="166" formatCode="d/mm/yy;@"/>
+    <numFmt numFmtId="167" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
   <fonts count="15" x14ac:knownFonts="1">
     <font>
@@ -3538,7 +3545,7 @@
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="103">
+  <cellXfs count="105">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3744,6 +3751,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="9" applyNumberFormat="1"/>
+    <xf numFmtId="167" fontId="3" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -6578,7 +6591,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:AB147"/>
+  <dimension ref="A1:AC147"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1796875" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.7265625" style="87" customWidth="1"/>
@@ -6593,11 +6606,11 @@
     <col min="15" max="15" width="10.26953125" style="91" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="10.26953125" style="91" customWidth="1"/>
     <col min="17" max="18" width="9.1796875" style="12"/>
-    <col min="19" max="20" width="12.08984375" style="12" customWidth="1"/>
-    <col min="21" max="16384" width="9.1796875" style="12"/>
+    <col min="20" max="21" width="12.08984375" style="12" customWidth="1"/>
+    <col min="22" max="16384" width="9.1796875" style="12"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" s="3" customFormat="1" ht="38.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:29" s="3" customFormat="1" ht="38.5" x14ac:dyDescent="0.35">
       <c r="A1" s="86" t="s">
         <v>1047</v>
       </c>
@@ -6649,26 +6662,31 @@
       <c r="Q1" s="93" t="s">
         <v>1049</v>
       </c>
-      <c r="R1" s="10" t="s">
+      <c r="R1" s="93" t="s">
+        <v>1066</v>
+      </c>
+      <c r="S1" s="93" t="s">
         <v>1050</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>1051</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>1063</v>
       </c>
-      <c r="U1" s="1"/>
-      <c r="V1" s="1"/>
+      <c r="V1" s="1" t="s">
+        <v>1067</v>
+      </c>
       <c r="W1" s="1"/>
       <c r="X1" s="1"/>
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
       <c r="AA1" s="1"/>
       <c r="AB1" s="1"/>
-    </row>
-    <row r="2" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="88" t="s">
+      <c r="AC1" s="1"/>
+    </row>
+    <row r="2" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="95" t="s">
         <v>850</v>
       </c>
       <c r="B2" s="88">
@@ -6719,16 +6737,18 @@
       <c r="Q2" s="92">
         <v>1.88</v>
       </c>
-      <c r="R2" s="11">
+      <c r="R2" s="92">
         <v>48.91</v>
       </c>
-      <c r="S2" s="11">
+      <c r="S2">
+        <v>98.1</v>
+      </c>
+      <c r="T2" s="11">
         <v>4673.7020000000002</v>
       </c>
-      <c r="T2" s="11">
+      <c r="U2" s="11">
         <v>17542.254883000001</v>
       </c>
-      <c r="U2" s="11"/>
       <c r="V2" s="11"/>
       <c r="W2" s="11"/>
       <c r="X2" s="11"/>
@@ -6736,9 +6756,10 @@
       <c r="Z2" s="11"/>
       <c r="AA2" s="11"/>
       <c r="AB2" s="11"/>
-    </row>
-    <row r="3" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="89" t="s">
+      <c r="AC2" s="11"/>
+    </row>
+    <row r="3" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="96" t="s">
         <v>851</v>
       </c>
       <c r="B3" s="89">
@@ -6789,16 +6810,18 @@
       <c r="Q3" s="92">
         <v>1.98</v>
       </c>
-      <c r="R3" s="11">
+      <c r="R3" s="92">
         <v>48.14</v>
       </c>
-      <c r="S3" s="11">
+      <c r="S3">
+        <v>95.4</v>
+      </c>
+      <c r="T3" s="11">
         <v>4854.2560000000003</v>
       </c>
-      <c r="T3" s="11">
+      <c r="U3" s="11">
         <v>17945.41200631579</v>
       </c>
-      <c r="U3" s="11"/>
       <c r="V3" s="11"/>
       <c r="W3" s="11"/>
       <c r="X3" s="11"/>
@@ -6806,9 +6829,10 @@
       <c r="Z3" s="11"/>
       <c r="AA3" s="11"/>
       <c r="AB3" s="11"/>
-    </row>
-    <row r="4" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="88" t="s">
+      <c r="AC3" s="11"/>
+    </row>
+    <row r="4" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="95" t="s">
         <v>852</v>
       </c>
       <c r="B4" s="88">
@@ -6859,16 +6883,18 @@
       <c r="Q4" s="92">
         <v>2.04</v>
       </c>
-      <c r="R4" s="11">
+      <c r="R4" s="92">
         <v>54.35</v>
       </c>
-      <c r="S4" s="11">
+      <c r="S4">
+        <v>93</v>
+      </c>
+      <c r="T4" s="11">
         <v>4938.01</v>
       </c>
-      <c r="T4" s="11">
+      <c r="U4" s="11">
         <v>17931.74502863636</v>
       </c>
-      <c r="U4" s="11"/>
       <c r="V4" s="11"/>
       <c r="W4" s="11"/>
       <c r="X4" s="11"/>
@@ -6876,9 +6902,10 @@
       <c r="Z4" s="11"/>
       <c r="AA4" s="11"/>
       <c r="AB4" s="11"/>
-    </row>
-    <row r="5" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="89" t="s">
+      <c r="AC4" s="11"/>
+    </row>
+    <row r="5" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="96" t="s">
         <v>853</v>
       </c>
       <c r="B5" s="89">
@@ -6929,16 +6956,18 @@
       <c r="Q5" s="92">
         <v>1.94</v>
       </c>
-      <c r="R5" s="11">
+      <c r="R5" s="92">
         <v>54.93</v>
       </c>
-      <c r="S5" s="11">
+      <c r="S5">
+        <v>95.9</v>
+      </c>
+      <c r="T5" s="11">
         <v>4985.951</v>
       </c>
-      <c r="T5" s="11">
+      <c r="U5" s="11">
         <v>17970.51320714286</v>
       </c>
-      <c r="U5" s="11"/>
       <c r="V5" s="11"/>
       <c r="W5" s="11"/>
       <c r="X5" s="11"/>
@@ -6946,9 +6975,10 @@
       <c r="Z5" s="11"/>
       <c r="AA5" s="11"/>
       <c r="AB5" s="11"/>
-    </row>
-    <row r="6" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="88" t="s">
+      <c r="AC5" s="11"/>
+    </row>
+    <row r="6" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="95" t="s">
         <v>854</v>
       </c>
       <c r="B6" s="88">
@@ -6999,16 +7029,18 @@
       <c r="Q6" s="92">
         <v>2.2000000000000002</v>
       </c>
-      <c r="R6" s="11">
+      <c r="R6" s="92">
         <v>53.76</v>
       </c>
-      <c r="S6" s="11">
+      <c r="S6">
+        <v>90.7</v>
+      </c>
+      <c r="T6" s="11">
         <v>5029.4319999999998</v>
       </c>
-      <c r="T6" s="11">
+      <c r="U6" s="11">
         <v>18124.713086</v>
       </c>
-      <c r="U6" s="11"/>
       <c r="V6" s="11"/>
       <c r="W6" s="11"/>
       <c r="X6" s="11"/>
@@ -7016,9 +7048,10 @@
       <c r="Z6" s="11"/>
       <c r="AA6" s="11"/>
       <c r="AB6" s="11"/>
-    </row>
-    <row r="7" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="89" t="s">
+      <c r="AC6" s="11"/>
+    </row>
+    <row r="7" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="96" t="s">
         <v>855</v>
       </c>
       <c r="B7" s="89">
@@ -7069,16 +7102,18 @@
       <c r="Q7" s="92">
         <v>2.36</v>
       </c>
-      <c r="R7" s="11">
+      <c r="R7" s="92">
         <v>55</v>
       </c>
-      <c r="S7" s="11">
+      <c r="S7">
+        <v>96.1</v>
+      </c>
+      <c r="T7" s="11">
         <v>5073.0420000000004</v>
       </c>
-      <c r="T7" s="11">
+      <c r="U7" s="11">
         <v>17927.21892727273</v>
       </c>
-      <c r="U7" s="11"/>
       <c r="V7" s="11"/>
       <c r="W7" s="11"/>
       <c r="X7" s="11"/>
@@ -7086,9 +7121,10 @@
       <c r="Z7" s="11"/>
       <c r="AA7" s="11"/>
       <c r="AB7" s="11"/>
-    </row>
-    <row r="8" spans="1:28" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="88" t="s">
+      <c r="AC7" s="11"/>
+    </row>
+    <row r="8" spans="1:29" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="95" t="s">
         <v>856</v>
       </c>
       <c r="B8" s="88">
@@ -7139,16 +7175,18 @@
       <c r="Q8" s="92">
         <v>2.3199999999999998</v>
       </c>
-      <c r="R8" s="11">
+      <c r="R8" s="92">
         <v>56</v>
       </c>
-      <c r="S8" s="11">
+      <c r="S8">
+        <v>93.1</v>
+      </c>
+      <c r="T8" s="11">
         <v>5082.8100000000004</v>
       </c>
-      <c r="T8" s="11">
+      <c r="U8" s="11">
         <v>17795.016602727272</v>
       </c>
-      <c r="U8" s="11"/>
       <c r="V8" s="11"/>
       <c r="W8" s="11"/>
       <c r="X8" s="11"/>
@@ -7156,9 +7194,10 @@
       <c r="Z8" s="11"/>
       <c r="AA8" s="11"/>
       <c r="AB8" s="11"/>
-    </row>
-    <row r="9" spans="1:28" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="89" t="s">
+      <c r="AC8" s="11"/>
+    </row>
+    <row r="9" spans="1:29" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="96" t="s">
         <v>857</v>
       </c>
       <c r="B9" s="89">
@@ -7209,18 +7248,21 @@
       <c r="Q9" s="92">
         <v>2.17</v>
       </c>
-      <c r="R9" s="11">
+      <c r="R9" s="92">
         <v>53.33</v>
       </c>
-      <c r="S9" s="11">
+      <c r="S9">
+        <v>91.9</v>
+      </c>
+      <c r="T9" s="11">
         <v>4934.6229999999996</v>
       </c>
-      <c r="T9" s="11">
+      <c r="U9" s="11">
         <v>17061.59323857143</v>
       </c>
     </row>
-    <row r="10" spans="1:28" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="88" t="s">
+    <row r="10" spans="1:29" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="95" t="s">
         <v>858</v>
       </c>
       <c r="B10" s="88">
@@ -7271,18 +7313,21 @@
       <c r="Q10" s="92">
         <v>2.17</v>
       </c>
-      <c r="R10" s="11">
+      <c r="R10" s="92">
         <v>56.96</v>
       </c>
-      <c r="S10" s="11">
+      <c r="S10">
+        <v>87.2</v>
+      </c>
+      <c r="T10" s="11">
         <v>4748.0039999999999</v>
       </c>
-      <c r="T10" s="11">
+      <c r="U10" s="11">
         <v>16339.949869523811</v>
       </c>
     </row>
-    <row r="11" spans="1:28" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="89" t="s">
+    <row r="11" spans="1:29" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="96" t="s">
         <v>859</v>
       </c>
       <c r="B11" s="89">
@@ -7333,18 +7378,21 @@
       <c r="Q11" s="92">
         <v>2.0699999999999998</v>
       </c>
-      <c r="R11" s="11">
+      <c r="R11" s="92">
         <v>56</v>
       </c>
-      <c r="S11" s="11">
+      <c r="S11">
+        <v>90</v>
+      </c>
+      <c r="T11" s="11">
         <v>4879.0370000000003</v>
       </c>
-      <c r="T11" s="11">
+      <c r="U11" s="11">
         <v>17182.282049545451</v>
       </c>
     </row>
-    <row r="12" spans="1:28" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="88" t="s">
+    <row r="12" spans="1:29" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="95" t="s">
         <v>860</v>
       </c>
       <c r="B12" s="88">
@@ -7395,18 +7443,21 @@
       <c r="Q12" s="92">
         <v>2.2599999999999998</v>
       </c>
-      <c r="R12" s="11">
+      <c r="R12" s="92">
         <v>58.4</v>
       </c>
-      <c r="S12" s="11">
+      <c r="S12">
+        <v>91.3</v>
+      </c>
+      <c r="T12" s="11">
         <v>5082.5079999999998</v>
       </c>
-      <c r="T12" s="11">
+      <c r="U12" s="11">
         <v>17724.513673000001</v>
       </c>
     </row>
-    <row r="13" spans="1:28" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="89" t="s">
+    <row r="13" spans="1:29" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="96" t="s">
         <v>861</v>
       </c>
       <c r="B13" s="89">
@@ -7457,18 +7508,21 @@
       <c r="Q13" s="92">
         <v>2.2400000000000002</v>
       </c>
-      <c r="R13" s="11">
+      <c r="R13" s="92">
         <v>51.99</v>
       </c>
-      <c r="S13" s="11">
+      <c r="S13">
+        <v>92.6</v>
+      </c>
+      <c r="T13" s="11">
         <v>5040.54</v>
       </c>
-      <c r="T13" s="11">
+      <c r="U13" s="11">
         <v>17542.854936363641</v>
       </c>
     </row>
-    <row r="14" spans="1:28" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="88" t="s">
+    <row r="14" spans="1:29" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="95" t="s">
         <v>862</v>
       </c>
       <c r="B14" s="88">
@@ -7519,18 +7573,21 @@
       <c r="Q14" s="92">
         <v>2.09</v>
       </c>
-      <c r="R14" s="11">
+      <c r="R14" s="92">
         <v>52.95</v>
       </c>
-      <c r="S14" s="11">
+      <c r="S14">
+        <v>92</v>
+      </c>
+      <c r="T14" s="11">
         <v>4610.7139999999999</v>
       </c>
-      <c r="T14" s="11">
+      <c r="U14" s="11">
         <v>16305.252107894739</v>
       </c>
     </row>
-    <row r="15" spans="1:28" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="89" t="s">
+    <row r="15" spans="1:29" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="96" t="s">
         <v>863</v>
       </c>
       <c r="B15" s="89">
@@ -7581,18 +7638,21 @@
       <c r="Q15" s="92">
         <v>1.78</v>
       </c>
-      <c r="R15" s="11">
+      <c r="R15" s="92">
         <v>46.38</v>
       </c>
-      <c r="S15" s="11">
+      <c r="S15">
+        <v>91.7</v>
+      </c>
+      <c r="T15" s="11">
         <v>4463.2060000000001</v>
       </c>
-      <c r="T15" s="11">
+      <c r="U15" s="11">
         <v>16299.8984375</v>
       </c>
     </row>
-    <row r="16" spans="1:28" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="88" t="s">
+    <row r="16" spans="1:29" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="95" t="s">
         <v>864</v>
       </c>
       <c r="B16" s="88">
@@ -7643,18 +7703,21 @@
       <c r="Q16" s="92">
         <v>1.89</v>
       </c>
-      <c r="R16" s="11">
+      <c r="R16" s="92">
         <v>46.38</v>
       </c>
-      <c r="S16" s="11">
+      <c r="S16">
+        <v>91</v>
+      </c>
+      <c r="T16" s="11">
         <v>4754.4790000000003</v>
       </c>
-      <c r="T16" s="11">
+      <c r="U16" s="11">
         <v>17302.142756363639</v>
       </c>
     </row>
-    <row r="17" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A17" s="89" t="s">
+    <row r="17" spans="1:21" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="96" t="s">
         <v>865</v>
       </c>
       <c r="B17" s="89">
@@ -7705,18 +7768,21 @@
       <c r="Q17" s="92">
         <v>1.81</v>
       </c>
-      <c r="R17" s="11">
+      <c r="R17" s="92">
         <v>46.14</v>
       </c>
-      <c r="S17" s="11">
+      <c r="S17">
+        <v>89</v>
+      </c>
+      <c r="T17" s="11">
         <v>4892.17</v>
       </c>
-      <c r="T17" s="11">
+      <c r="U17" s="11">
         <v>17844.365886190481</v>
       </c>
     </row>
-    <row r="18" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="88" t="s">
+    <row r="18" spans="1:21" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="95" t="s">
         <v>866</v>
       </c>
       <c r="B18" s="88">
@@ -7767,18 +7833,21 @@
       <c r="Q18" s="92">
         <v>1.81</v>
       </c>
-      <c r="R18" s="11">
+      <c r="R18" s="92">
         <v>44.06</v>
       </c>
-      <c r="S18" s="11">
+      <c r="S18">
+        <v>94.7</v>
+      </c>
+      <c r="T18" s="11">
         <v>4788.2349999999997</v>
       </c>
-      <c r="T18" s="11">
+      <c r="U18" s="11">
         <v>17692.320034285709</v>
       </c>
     </row>
-    <row r="19" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="89" t="s">
+    <row r="19" spans="1:21" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="96" t="s">
         <v>867</v>
       </c>
       <c r="B19" s="89">
@@ -7829,18 +7898,21 @@
       <c r="Q19" s="92">
         <v>1.64</v>
       </c>
-      <c r="R19" s="11">
+      <c r="R19" s="92">
         <v>44.95</v>
       </c>
-      <c r="S19" s="11">
+      <c r="S19">
+        <v>93.5</v>
+      </c>
+      <c r="T19" s="11">
         <v>4856.232</v>
       </c>
-      <c r="T19" s="11">
+      <c r="U19" s="11">
         <v>17754.867808636369</v>
       </c>
     </row>
-    <row r="20" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="88" t="s">
+    <row r="20" spans="1:21" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="95" t="s">
         <v>868</v>
       </c>
       <c r="B20" s="88">
@@ -7891,18 +7963,21 @@
       <c r="Q20" s="92">
         <v>1.5</v>
       </c>
-      <c r="R20" s="11">
+      <c r="R20" s="92">
         <v>45.82</v>
       </c>
-      <c r="S20" s="11">
+      <c r="S20">
+        <v>90</v>
+      </c>
+      <c r="T20" s="11">
         <v>5023.9889999999996</v>
       </c>
-      <c r="T20" s="11">
+      <c r="U20" s="11">
         <v>18341.182422000002</v>
       </c>
     </row>
-    <row r="21" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="89" t="s">
+    <row r="21" spans="1:21" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="96" t="s">
         <v>869</v>
       </c>
       <c r="B21" s="89">
@@ -7953,18 +8028,21 @@
       <c r="Q21" s="92">
         <v>1.56</v>
       </c>
-      <c r="R21" s="11">
+      <c r="R21" s="92">
         <v>45.44</v>
       </c>
-      <c r="S21" s="11">
+      <c r="S21">
+        <v>89.8</v>
+      </c>
+      <c r="T21" s="11">
         <v>5217.0379999999996</v>
       </c>
-      <c r="T21" s="11">
+      <c r="U21" s="11">
         <v>18495.187499565222</v>
       </c>
     </row>
-    <row r="22" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="88" t="s">
+    <row r="22" spans="1:21" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="95" t="s">
         <v>870</v>
       </c>
       <c r="B22" s="88">
@@ -8015,18 +8093,21 @@
       <c r="Q22" s="92">
         <v>1.63</v>
       </c>
-      <c r="R22" s="11">
+      <c r="R22" s="92">
         <v>46.6</v>
       </c>
-      <c r="S22" s="11">
+      <c r="S22">
+        <v>91.2</v>
+      </c>
+      <c r="T22" s="11">
         <v>5254.1540000000005</v>
       </c>
-      <c r="T22" s="11">
+      <c r="U22" s="11">
         <v>18267.402995238099</v>
       </c>
     </row>
-    <row r="23" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="89" t="s">
+    <row r="23" spans="1:21" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="96" t="s">
         <v>871</v>
       </c>
       <c r="B23" s="89">
@@ -8077,18 +8158,21 @@
       <c r="Q23" s="92">
         <v>1.76</v>
       </c>
-      <c r="R23" s="11">
+      <c r="R23" s="92">
         <v>45.36</v>
       </c>
-      <c r="S23" s="11">
+      <c r="S23">
+        <v>87.2</v>
+      </c>
+      <c r="T23" s="11">
         <v>5255.9889999999996</v>
       </c>
-      <c r="T23" s="11">
+      <c r="U23" s="11">
         <v>18184.546409999999</v>
       </c>
     </row>
-    <row r="24" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="88" t="s">
+    <row r="24" spans="1:21" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="95" t="s">
         <v>872</v>
       </c>
       <c r="B24" s="88">
@@ -8139,18 +8223,21 @@
       <c r="Q24" s="92">
         <v>2.14</v>
       </c>
-      <c r="R24" s="11">
+      <c r="R24" s="92">
         <v>49.13</v>
       </c>
-      <c r="S24" s="11">
+      <c r="S24">
+        <v>93.8</v>
+      </c>
+      <c r="T24" s="11">
         <v>5260.5649999999996</v>
       </c>
-      <c r="T24" s="11">
+      <c r="U24" s="11">
         <v>18697.326637619051</v>
       </c>
     </row>
-    <row r="25" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="89" t="s">
+    <row r="25" spans="1:21" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="96" t="s">
         <v>873</v>
       </c>
       <c r="B25" s="89">
@@ -8201,18 +8288,21 @@
       <c r="Q25" s="92">
         <v>2.4900000000000002</v>
       </c>
-      <c r="R25" s="11">
+      <c r="R25" s="92">
         <v>46.28</v>
       </c>
-      <c r="S25" s="11">
+      <c r="S25">
+        <v>98.2</v>
+      </c>
+      <c r="T25" s="11">
         <v>5413.1170000000002</v>
       </c>
-      <c r="T25" s="11">
+      <c r="U25" s="11">
         <v>19712.423736190471</v>
       </c>
     </row>
-    <row r="26" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="88" t="s">
+    <row r="26" spans="1:21" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="95" t="s">
         <v>874</v>
       </c>
       <c r="B26" s="88">
@@ -8263,18 +8353,21 @@
       <c r="Q26" s="92">
         <v>2.4300000000000002</v>
       </c>
-      <c r="R26" s="11">
+      <c r="R26" s="92">
         <v>45.49</v>
       </c>
-      <c r="S26" s="11">
+      <c r="S26">
+        <v>98.5</v>
+      </c>
+      <c r="T26" s="11">
         <v>5561.424</v>
       </c>
-      <c r="T26" s="11">
+      <c r="U26" s="11">
         <v>19908.152539999999</v>
       </c>
     </row>
-    <row r="27" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="89" t="s">
+    <row r="27" spans="1:21" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="96" t="s">
         <v>875</v>
       </c>
       <c r="B27" s="89">
@@ -8325,18 +8418,21 @@
       <c r="Q27" s="92">
         <v>2.42</v>
       </c>
-      <c r="R27" s="11">
+      <c r="R27" s="92">
         <v>41.96</v>
       </c>
-      <c r="S27" s="11">
+      <c r="S27">
+        <v>96.3</v>
+      </c>
+      <c r="T27" s="11">
         <v>5764.7020000000002</v>
       </c>
-      <c r="T27" s="11">
+      <c r="U27" s="11">
         <v>20424.144120000001</v>
       </c>
     </row>
-    <row r="28" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="88" t="s">
+    <row r="28" spans="1:21" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="95" t="s">
         <v>876</v>
       </c>
       <c r="B28" s="88">
@@ -8387,18 +8483,21 @@
       <c r="Q28" s="92">
         <v>2.48</v>
       </c>
-      <c r="R28" s="11">
+      <c r="R28" s="92">
         <v>43.94</v>
       </c>
-      <c r="S28" s="11">
+      <c r="S28">
+        <v>96.9</v>
+      </c>
+      <c r="T28" s="11">
         <v>5864.9639999999999</v>
       </c>
-      <c r="T28" s="11">
+      <c r="U28" s="11">
         <v>20823.05799913044</v>
       </c>
     </row>
-    <row r="29" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="89" t="s">
+    <row r="29" spans="1:21" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="96" t="s">
         <v>877</v>
       </c>
       <c r="B29" s="89">
@@ -8449,18 +8548,21 @@
       <c r="Q29" s="92">
         <v>2.2999999999999998</v>
       </c>
-      <c r="R29" s="11">
+      <c r="R29" s="92">
         <v>50.39</v>
       </c>
-      <c r="S29" s="11">
+      <c r="S29">
+        <v>97</v>
+      </c>
+      <c r="T29" s="11">
         <v>5912.1689999999999</v>
       </c>
-      <c r="T29" s="11">
+      <c r="U29" s="11">
         <v>20684.693668421049</v>
       </c>
     </row>
-    <row r="30" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="88" t="s">
+    <row r="30" spans="1:21" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="95" t="s">
         <v>878</v>
       </c>
       <c r="B30" s="88">
@@ -8511,18 +8613,21 @@
       <c r="Q30" s="92">
         <v>2.2999999999999998</v>
       </c>
-      <c r="R30" s="11">
+      <c r="R30" s="92">
         <v>49.64</v>
       </c>
-      <c r="S30" s="11">
+      <c r="S30">
+        <v>97.1</v>
+      </c>
+      <c r="T30" s="11">
         <v>6124.8779999999997</v>
       </c>
-      <c r="T30" s="11">
+      <c r="U30" s="11">
         <v>20936.81125772727</v>
       </c>
     </row>
-    <row r="31" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="89" t="s">
+    <row r="31" spans="1:21" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="96" t="s">
         <v>879</v>
       </c>
       <c r="B31" s="89">
@@ -8573,18 +8678,21 @@
       <c r="Q31" s="92">
         <v>2.19</v>
       </c>
-      <c r="R31" s="11">
+      <c r="R31" s="92">
         <v>45.06</v>
       </c>
-      <c r="S31" s="11">
+      <c r="S31">
+        <v>95</v>
+      </c>
+      <c r="T31" s="11">
         <v>6224.2860000000001</v>
       </c>
-      <c r="T31" s="11">
+      <c r="U31" s="11">
         <v>21317.79536636364</v>
       </c>
     </row>
-    <row r="32" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="88" t="s">
+    <row r="32" spans="1:21" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="95" t="s">
         <v>880</v>
       </c>
       <c r="B32" s="88">
@@ -8635,18 +8743,21 @@
       <c r="Q32" s="92">
         <v>2.3199999999999998</v>
       </c>
-      <c r="R32" s="11">
+      <c r="R32" s="92">
         <v>43.48</v>
       </c>
-      <c r="S32" s="11">
+      <c r="S32">
+        <v>93.4</v>
+      </c>
+      <c r="T32" s="11">
         <v>6294.674</v>
       </c>
-      <c r="T32" s="11">
+      <c r="U32" s="11">
         <v>21581.250975999999</v>
       </c>
     </row>
-    <row r="33" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="89" t="s">
+    <row r="33" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="96" t="s">
         <v>881</v>
       </c>
       <c r="B33" s="89">
@@ -8697,18 +8808,21 @@
       <c r="Q33" s="92">
         <v>2.21</v>
       </c>
-      <c r="R33" s="11">
+      <c r="R33" s="92">
         <v>50.23</v>
       </c>
-      <c r="S33" s="11">
+      <c r="S33">
+        <v>96.8</v>
+      </c>
+      <c r="T33" s="11">
         <v>6311.3969999999999</v>
       </c>
-      <c r="T33" s="11">
+      <c r="U33" s="11">
         <v>21914.07693608696</v>
       </c>
     </row>
-    <row r="34" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="88" t="s">
+    <row r="34" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="95" t="s">
         <v>882</v>
       </c>
       <c r="B34" s="88">
@@ -8759,18 +8873,21 @@
       <c r="Q34" s="92">
         <v>2.2000000000000002</v>
       </c>
-      <c r="R34" s="11">
+      <c r="R34" s="92">
         <v>53.79</v>
       </c>
-      <c r="S34" s="11">
+      <c r="S34">
+        <v>95.1</v>
+      </c>
+      <c r="T34" s="11">
         <v>6428.0789999999997</v>
       </c>
-      <c r="T34" s="11">
+      <c r="U34" s="11">
         <v>22173.413965</v>
       </c>
     </row>
-    <row r="35" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="89" t="s">
+    <row r="35" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="96" t="s">
         <v>883</v>
       </c>
       <c r="B35" s="89">
@@ -8821,18 +8938,21 @@
       <c r="Q35" s="92">
         <v>2.36</v>
       </c>
-      <c r="R35" s="11">
+      <c r="R35" s="92">
         <v>56.16</v>
       </c>
-      <c r="S35" s="11">
+      <c r="S35">
+        <v>100.7</v>
+      </c>
+      <c r="T35" s="11">
         <v>6603.0110000000004</v>
       </c>
-      <c r="T35" s="11">
+      <c r="U35" s="11">
         <v>23036.237394090909</v>
       </c>
     </row>
-    <row r="36" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="88" t="s">
+    <row r="36" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="95" t="s">
         <v>884</v>
       </c>
       <c r="B36" s="88">
@@ -8883,18 +9003,21 @@
       <c r="Q36" s="92">
         <v>2.35</v>
       </c>
-      <c r="R36" s="11">
+      <c r="R36" s="92">
         <v>54.56</v>
       </c>
-      <c r="S36" s="11">
+      <c r="S36">
+        <v>98.5</v>
+      </c>
+      <c r="T36" s="11">
         <v>6796.0429999999997</v>
       </c>
-      <c r="T36" s="11">
+      <c r="U36" s="11">
         <v>23557.929409523811</v>
       </c>
     </row>
-    <row r="37" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="89" t="s">
+    <row r="37" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="96" t="s">
         <v>885</v>
       </c>
       <c r="B37" s="89">
@@ -8945,18 +9068,21 @@
       <c r="Q37" s="92">
         <v>2.4</v>
       </c>
-      <c r="R37" s="11">
+      <c r="R37" s="92">
         <v>47.87</v>
       </c>
-      <c r="S37" s="11">
+      <c r="S37">
+        <v>95.9</v>
+      </c>
+      <c r="T37" s="11">
         <v>6889.741</v>
       </c>
-      <c r="T37" s="11">
+      <c r="U37" s="11">
         <v>24545.384180500001</v>
       </c>
     </row>
-    <row r="38" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="88" t="s">
+    <row r="38" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="95" t="s">
         <v>886</v>
       </c>
       <c r="B38" s="88">
@@ -9007,18 +9133,21 @@
       <c r="Q38" s="92">
         <v>2.58</v>
       </c>
-      <c r="R38" s="11">
+      <c r="R38" s="92">
         <v>47.1</v>
       </c>
-      <c r="S38" s="11">
+      <c r="S38">
+        <v>95.7</v>
+      </c>
+      <c r="T38" s="11">
         <v>7279.4979999999996</v>
       </c>
-      <c r="T38" s="11">
+      <c r="U38" s="11">
         <v>25804.017765238099</v>
       </c>
     </row>
-    <row r="39" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="89" t="s">
+    <row r="39" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="96" t="s">
         <v>887</v>
       </c>
       <c r="B39" s="89">
@@ -9069,18 +9198,21 @@
       <c r="Q39" s="92">
         <v>2.86</v>
       </c>
-      <c r="R39" s="11">
+      <c r="R39" s="92">
         <v>45.9</v>
       </c>
-      <c r="S39" s="11">
+      <c r="S39">
+        <v>99.7</v>
+      </c>
+      <c r="T39" s="11">
         <v>7161.7730000000001</v>
       </c>
-      <c r="T39" s="11">
+      <c r="U39" s="11">
         <v>24981.545230526321</v>
       </c>
     </row>
-    <row r="40" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A40" s="88" t="s">
+    <row r="40" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="95" t="s">
         <v>888</v>
       </c>
       <c r="B40" s="88">
@@ -9131,18 +9263,21 @@
       <c r="Q40" s="92">
         <v>2.84</v>
       </c>
-      <c r="R40" s="11">
+      <c r="R40" s="92">
         <v>44.62</v>
       </c>
-      <c r="S40" s="11">
+      <c r="S40">
+        <v>101.4</v>
+      </c>
+      <c r="T40" s="11">
         <v>7311.5060000000003</v>
       </c>
-      <c r="T40" s="11">
+      <c r="U40" s="11">
         <v>24582.17038904762</v>
       </c>
     </row>
-    <row r="41" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="89" t="s">
+    <row r="41" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="96" t="s">
         <v>889</v>
       </c>
       <c r="B41" s="89">
@@ -9193,18 +9328,21 @@
       <c r="Q41" s="92">
         <v>2.87</v>
       </c>
-      <c r="R41" s="11">
+      <c r="R41" s="92">
         <v>45.14</v>
       </c>
-      <c r="S41" s="11">
+      <c r="S41">
+        <v>98.8</v>
+      </c>
+      <c r="T41" s="11">
         <v>7084.1419999999998</v>
       </c>
-      <c r="T41" s="11">
+      <c r="U41" s="11">
         <v>24304.212890476188</v>
       </c>
     </row>
-    <row r="42" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A42" s="88" t="s">
+    <row r="42" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="95" t="s">
         <v>890</v>
       </c>
       <c r="B42" s="88">
@@ -9255,18 +9393,21 @@
       <c r="Q42" s="92">
         <v>2.98</v>
       </c>
-      <c r="R42" s="11">
+      <c r="R42" s="92">
         <v>38.29</v>
       </c>
-      <c r="S42" s="11">
+      <c r="S42">
+        <v>98</v>
+      </c>
+      <c r="T42" s="11">
         <v>7339.3270000000002</v>
       </c>
-      <c r="T42" s="11">
+      <c r="U42" s="11">
         <v>24572.532227272732</v>
       </c>
     </row>
-    <row r="43" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A43" s="89" t="s">
+    <row r="43" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A43" s="96" t="s">
         <v>891</v>
       </c>
       <c r="B43" s="89">
@@ -9317,18 +9458,21 @@
       <c r="Q43" s="92">
         <v>2.91</v>
       </c>
-      <c r="R43" s="11">
+      <c r="R43" s="92">
         <v>36.979999999999997</v>
       </c>
-      <c r="S43" s="11">
+      <c r="S43">
+        <v>98.2</v>
+      </c>
+      <c r="T43" s="11">
         <v>7645.1390000000001</v>
       </c>
-      <c r="T43" s="11">
+      <c r="U43" s="11">
         <v>24790.108353333329</v>
       </c>
     </row>
-    <row r="44" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A44" s="88" t="s">
+    <row r="44" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="95" t="s">
         <v>892</v>
       </c>
       <c r="B44" s="88">
@@ -9379,18 +9523,21 @@
       <c r="Q44" s="92">
         <v>2.89</v>
       </c>
-      <c r="R44" s="11">
+      <c r="R44" s="92">
         <v>37.07</v>
       </c>
-      <c r="S44" s="11">
+      <c r="S44">
+        <v>97.9</v>
+      </c>
+      <c r="T44" s="11">
         <v>7756.8639999999996</v>
       </c>
-      <c r="T44" s="11">
+      <c r="U44" s="11">
         <v>24978.231306190479</v>
       </c>
     </row>
-    <row r="45" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A45" s="89" t="s">
+    <row r="45" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="96" t="s">
         <v>893</v>
       </c>
       <c r="B45" s="89">
@@ -9441,18 +9588,21 @@
       <c r="Q45" s="92">
         <v>2.89</v>
       </c>
-      <c r="R45" s="11">
+      <c r="R45" s="92">
         <v>38.450000000000003</v>
       </c>
-      <c r="S45" s="11">
+      <c r="S45">
+        <v>96.2</v>
+      </c>
+      <c r="T45" s="11">
         <v>7892.2330000000002</v>
       </c>
-      <c r="T45" s="11">
+      <c r="U45" s="11">
         <v>25629.98828173913</v>
       </c>
     </row>
-    <row r="46" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A46" s="88" t="s">
+    <row r="46" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="95" t="s">
         <v>894</v>
       </c>
       <c r="B46" s="88">
@@ -9503,18 +9653,24 @@
       <c r="Q46" s="92">
         <v>3</v>
       </c>
-      <c r="R46" s="11">
+      <c r="R46" s="92">
         <v>35.26</v>
       </c>
-      <c r="S46" s="11">
+      <c r="S46">
+        <v>100.1</v>
+      </c>
+      <c r="T46" s="11">
         <v>7983.3069999999998</v>
       </c>
-      <c r="T46" s="11">
+      <c r="U46" s="11">
         <v>26232.667968947371</v>
       </c>
-    </row>
-    <row r="47" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A47" s="89" t="s">
+      <c r="V46" s="11">
+        <v>102.84</v>
+      </c>
+    </row>
+    <row r="47" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="96" t="s">
         <v>895</v>
       </c>
       <c r="B47" s="89">
@@ -9565,18 +9721,24 @@
       <c r="Q47" s="92">
         <v>3.15</v>
       </c>
-      <c r="R47" s="11">
+      <c r="R47" s="92">
         <v>35.1</v>
       </c>
-      <c r="S47" s="11">
+      <c r="S47">
+        <v>98.6</v>
+      </c>
+      <c r="T47" s="11">
         <v>7527.0839999999998</v>
       </c>
-      <c r="T47" s="11">
+      <c r="U47" s="11">
         <v>25609.341882173911</v>
       </c>
-    </row>
-    <row r="48" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A48" s="88" t="s">
+      <c r="V47" s="11">
+        <v>104.74</v>
+      </c>
+    </row>
+    <row r="48" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A48" s="95" t="s">
         <v>896</v>
       </c>
       <c r="B48" s="88">
@@ -9627,18 +9789,24 @@
       <c r="Q48" s="92">
         <v>3.12</v>
       </c>
-      <c r="R48" s="11">
+      <c r="R48" s="92">
         <v>35.4</v>
       </c>
-      <c r="S48" s="11">
+      <c r="S48">
+        <v>97.5</v>
+      </c>
+      <c r="T48" s="11">
         <v>7236.0810000000001</v>
       </c>
-      <c r="T48" s="11">
+      <c r="U48" s="11">
         <v>25258.675315714281</v>
       </c>
-    </row>
-    <row r="49" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A49" s="89" t="s">
+      <c r="V48" s="11">
+        <v>106.95</v>
+      </c>
+    </row>
+    <row r="49" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A49" s="96" t="s">
         <v>897</v>
       </c>
       <c r="B49" s="89">
@@ -9689,18 +9857,24 @@
       <c r="Q49" s="92">
         <v>2.83</v>
       </c>
-      <c r="R49" s="11">
+      <c r="R49" s="92">
         <v>39</v>
       </c>
-      <c r="S49" s="11">
+      <c r="S49">
+        <v>98.3</v>
+      </c>
+      <c r="T49" s="11">
         <v>6814.2920000000004</v>
       </c>
-      <c r="T49" s="11">
+      <c r="U49" s="11">
         <v>23805.545231052631</v>
       </c>
-    </row>
-    <row r="50" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="88" t="s">
+      <c r="V49" s="11">
+        <v>109.83</v>
+      </c>
+    </row>
+    <row r="50" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A50" s="95" t="s">
         <v>898</v>
       </c>
       <c r="B50" s="88">
@@ -9751,18 +9925,24 @@
       <c r="Q50" s="92">
         <v>2.71</v>
       </c>
-      <c r="R50" s="11">
+      <c r="R50" s="92">
         <v>32.17</v>
       </c>
-      <c r="S50" s="11">
+      <c r="S50">
+        <v>91.2</v>
+      </c>
+      <c r="T50" s="11">
         <v>6979.6559999999999</v>
       </c>
-      <c r="T50" s="11">
+      <c r="U50" s="11">
         <v>24157.795107619051</v>
       </c>
-    </row>
-    <row r="51" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A51" s="89" t="s">
+      <c r="V50" s="11">
+        <v>111.16</v>
+      </c>
+    </row>
+    <row r="51" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A51" s="96" t="s">
         <v>899</v>
       </c>
       <c r="B51" s="89">
@@ -9813,18 +9993,24 @@
       <c r="Q51" s="92">
         <v>2.68</v>
       </c>
-      <c r="R51" s="11">
+      <c r="R51" s="92">
         <v>38.85</v>
       </c>
-      <c r="S51" s="11">
+      <c r="S51">
+        <v>93.8</v>
+      </c>
+      <c r="T51" s="11">
         <v>7430.0770000000002</v>
       </c>
-      <c r="T51" s="11">
+      <c r="U51" s="11">
         <v>25605.52683105263</v>
       </c>
-    </row>
-    <row r="52" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A52" s="88" t="s">
+      <c r="V51" s="11">
+        <v>113.74</v>
+      </c>
+    </row>
+    <row r="52" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A52" s="95" t="s">
         <v>900</v>
       </c>
       <c r="B52" s="88">
@@ -9875,18 +10061,24 @@
       <c r="Q52" s="92">
         <v>2.57</v>
       </c>
-      <c r="R52" s="11">
+      <c r="R52" s="92">
         <v>33.270000000000003</v>
       </c>
-      <c r="S52" s="11">
+      <c r="S52">
+        <v>98.4</v>
+      </c>
+      <c r="T52" s="11">
         <v>7629.3670000000002</v>
       </c>
-      <c r="T52" s="11">
+      <c r="U52" s="11">
         <v>25722.62118714286</v>
       </c>
-    </row>
-    <row r="53" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A53" s="89" t="s">
+      <c r="V52" s="11">
+        <v>118.27</v>
+      </c>
+    </row>
+    <row r="53" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A53" s="96" t="s">
         <v>901</v>
       </c>
       <c r="B53" s="89">
@@ -9937,18 +10129,24 @@
       <c r="Q53" s="92">
         <v>2.5299999999999998</v>
       </c>
-      <c r="R53" s="11">
+      <c r="R53" s="92">
         <v>35.04</v>
       </c>
-      <c r="S53" s="11">
+      <c r="S53">
+        <v>97.2</v>
+      </c>
+      <c r="T53" s="11">
         <v>7993.3689999999997</v>
       </c>
-      <c r="T53" s="11">
+      <c r="U53" s="11">
         <v>26401.577381428571</v>
       </c>
-    </row>
-    <row r="54" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="88" t="s">
+      <c r="V53" s="11">
+        <v>120.18</v>
+      </c>
+    </row>
+    <row r="54" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A54" s="95" t="s">
         <v>902</v>
       </c>
       <c r="B54" s="88">
@@ -9999,18 +10197,24 @@
       <c r="Q54" s="92">
         <v>2.4</v>
       </c>
-      <c r="R54" s="11">
+      <c r="R54" s="92">
         <v>39.35</v>
       </c>
-      <c r="S54" s="11">
+      <c r="S54">
+        <v>100</v>
+      </c>
+      <c r="T54" s="11">
         <v>7804.8209999999999</v>
       </c>
-      <c r="T54" s="11">
+      <c r="U54" s="11">
         <v>25744.788530000002</v>
       </c>
-    </row>
-    <row r="55" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="89" t="s">
+      <c r="V54" s="11">
+        <v>119.81</v>
+      </c>
+    </row>
+    <row r="55" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A55" s="96" t="s">
         <v>903</v>
       </c>
       <c r="B55" s="89">
@@ -10061,18 +10265,24 @@
       <c r="Q55" s="92">
         <v>2.0699999999999998</v>
       </c>
-      <c r="R55" s="11">
+      <c r="R55" s="92">
         <v>42.99</v>
       </c>
-      <c r="S55" s="11">
+      <c r="S55">
+        <v>98.2</v>
+      </c>
+      <c r="T55" s="11">
         <v>7825.4589999999998</v>
       </c>
-      <c r="T55" s="11">
+      <c r="U55" s="11">
         <v>26160.100879500002</v>
       </c>
-    </row>
-    <row r="56" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A56" s="88" t="s">
+      <c r="V55" s="11">
+        <v>120.23</v>
+      </c>
+    </row>
+    <row r="56" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A56" s="95" t="s">
         <v>904</v>
       </c>
       <c r="B56" s="88">
@@ -10123,18 +10333,24 @@
       <c r="Q56" s="92">
         <v>2.06</v>
       </c>
-      <c r="R56" s="11">
+      <c r="R56" s="92">
         <v>45.67</v>
       </c>
-      <c r="S56" s="11">
+      <c r="S56">
+        <v>98.4</v>
+      </c>
+      <c r="T56" s="11">
         <v>8205.5990000000002</v>
       </c>
-      <c r="T56" s="11">
+      <c r="U56" s="11">
         <v>27089.18670136364</v>
       </c>
-    </row>
-    <row r="57" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A57" s="89" t="s">
+      <c r="V56" s="11">
+        <v>120.89</v>
+      </c>
+    </row>
+    <row r="57" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A57" s="96" t="s">
         <v>905</v>
       </c>
       <c r="B57" s="89">
@@ -10185,18 +10401,24 @@
       <c r="Q57" s="92">
         <v>1.63</v>
       </c>
-      <c r="R57" s="11">
+      <c r="R57" s="92">
         <v>44.94</v>
       </c>
-      <c r="S57" s="11">
+      <c r="S57">
+        <v>89.8</v>
+      </c>
+      <c r="T57" s="11">
         <v>7910.933</v>
       </c>
-      <c r="T57" s="11">
+      <c r="U57" s="11">
         <v>26057.728071363639</v>
       </c>
-    </row>
-    <row r="58" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A58" s="88" t="s">
+      <c r="V57" s="11">
+        <v>119.9</v>
+      </c>
+    </row>
+    <row r="58" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A58" s="95" t="s">
         <v>906</v>
       </c>
       <c r="B58" s="88">
@@ -10247,18 +10469,24 @@
       <c r="Q58" s="92">
         <v>1.7</v>
       </c>
-      <c r="R58" s="11">
+      <c r="R58" s="92">
         <v>44.42</v>
       </c>
-      <c r="S58" s="11">
+      <c r="S58">
+        <v>93.2</v>
+      </c>
+      <c r="T58" s="11">
         <v>8087.7</v>
       </c>
-      <c r="T58" s="11">
+      <c r="U58" s="11">
         <v>26900.213964499999</v>
       </c>
-    </row>
-    <row r="59" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A59" s="89" t="s">
+      <c r="V58" s="11">
+        <v>118.5</v>
+      </c>
+    </row>
+    <row r="59" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A59" s="96" t="s">
         <v>907</v>
       </c>
       <c r="B59" s="89">
@@ -10309,18 +10537,24 @@
       <c r="Q59" s="92">
         <v>1.71</v>
       </c>
-      <c r="R59" s="11">
+      <c r="R59" s="92">
         <v>42.24</v>
       </c>
-      <c r="S59" s="11">
+      <c r="S59">
+        <v>95.5</v>
+      </c>
+      <c r="T59" s="11">
         <v>8079.2740000000003</v>
       </c>
-      <c r="T59" s="11">
+      <c r="U59" s="11">
         <v>26736.797724347831</v>
       </c>
-    </row>
-    <row r="60" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A60" s="88" t="s">
+      <c r="V59" s="11">
+        <v>116.48</v>
+      </c>
+    </row>
+    <row r="60" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A60" s="95" t="s">
         <v>908</v>
       </c>
       <c r="B60" s="88">
@@ -10371,18 +10605,24 @@
       <c r="Q60" s="92">
         <v>1.81</v>
       </c>
-      <c r="R60" s="11">
+      <c r="R60" s="92">
         <v>39.68</v>
       </c>
-      <c r="S60" s="11">
+      <c r="S60">
+        <v>96.8</v>
+      </c>
+      <c r="T60" s="11">
         <v>8517.5779999999995</v>
       </c>
-      <c r="T60" s="11">
+      <c r="U60" s="11">
         <v>27797.046093500001</v>
       </c>
-    </row>
-    <row r="61" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A61" s="89" t="s">
+      <c r="V60" s="11">
+        <v>113.78</v>
+      </c>
+    </row>
+    <row r="61" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A61" s="96" t="s">
         <v>909</v>
       </c>
       <c r="B61" s="89">
@@ -10433,18 +10673,24 @@
       <c r="Q61" s="92">
         <v>1.86</v>
       </c>
-      <c r="R61" s="11">
+      <c r="R61" s="92">
         <v>42.11</v>
       </c>
-      <c r="S61" s="11">
+      <c r="S61">
+        <v>99.3</v>
+      </c>
+      <c r="T61" s="11">
         <v>8778.5910000000003</v>
       </c>
-      <c r="T61" s="11">
+      <c r="U61" s="11">
         <v>28167.005767619052</v>
       </c>
-    </row>
-    <row r="62" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A62" s="88" t="s">
+      <c r="V61" s="11">
+        <v>113.46</v>
+      </c>
+    </row>
+    <row r="62" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A62" s="95" t="s">
         <v>910</v>
       </c>
       <c r="B62" s="88">
@@ -10495,18 +10741,24 @@
       <c r="Q62" s="92">
         <v>1.76</v>
       </c>
-      <c r="R62" s="11">
+      <c r="R62" s="92">
         <v>40.44</v>
       </c>
-      <c r="S62" s="11">
+      <c r="S62">
+        <v>99.8</v>
+      </c>
+      <c r="T62" s="11">
         <v>9233.36</v>
       </c>
-      <c r="T62" s="11">
+      <c r="U62" s="11">
         <v>28879.994326190481</v>
       </c>
-    </row>
-    <row r="63" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A63" s="89" t="s">
+      <c r="V62" s="11">
+        <v>114.1</v>
+      </c>
+    </row>
+    <row r="63" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A63" s="96" t="s">
         <v>911</v>
       </c>
       <c r="B63" s="89">
@@ -10557,18 +10809,24 @@
       <c r="Q63" s="92">
         <v>1.5</v>
       </c>
-      <c r="R63" s="11">
+      <c r="R63" s="92">
         <v>38.909999999999997</v>
       </c>
-      <c r="S63" s="11">
+      <c r="S63">
+        <v>101</v>
+      </c>
+      <c r="T63" s="11">
         <v>9418.8490000000002</v>
       </c>
-      <c r="T63" s="11">
+      <c r="U63" s="11">
         <v>28519.73160052632</v>
       </c>
-    </row>
-    <row r="64" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A64" s="88" t="s">
+      <c r="V63" s="11">
+        <v>114.17</v>
+      </c>
+    </row>
+    <row r="64" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A64" s="95" t="s">
         <v>912</v>
       </c>
       <c r="B64" s="88">
@@ -10619,18 +10877,24 @@
       <c r="Q64" s="92">
         <v>0.87</v>
       </c>
-      <c r="R64" s="11">
+      <c r="R64" s="92">
         <v>38.64</v>
       </c>
-      <c r="S64" s="11">
+      <c r="S64">
+        <v>89.1</v>
+      </c>
+      <c r="T64" s="11">
         <v>7772.2060000000001</v>
       </c>
-      <c r="T64" s="11">
+      <c r="U64" s="11">
         <v>22637.420810454551</v>
       </c>
-    </row>
-    <row r="65" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A65" s="89" t="s">
+      <c r="V64" s="11">
+        <v>114.57</v>
+      </c>
+    </row>
+    <row r="65" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A65" s="96" t="s">
         <v>913</v>
       </c>
       <c r="B65" s="89">
@@ -10681,18 +10945,24 @@
       <c r="Q65" s="92">
         <v>0.66</v>
       </c>
-      <c r="R65" s="11">
+      <c r="R65" s="92">
         <v>36.22</v>
       </c>
-      <c r="S65" s="11">
+      <c r="S65">
+        <v>71.8</v>
+      </c>
+      <c r="T65" s="11">
         <v>8292.4069999999992</v>
       </c>
-      <c r="T65" s="11">
+      <c r="U65" s="11">
         <v>23293.89983285714</v>
       </c>
-    </row>
-    <row r="66" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A66" s="88" t="s">
+      <c r="V65" s="11">
+        <v>114.67</v>
+      </c>
+    </row>
+    <row r="66" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A66" s="95" t="s">
         <v>914</v>
       </c>
       <c r="B66" s="88">
@@ -10743,18 +11013,24 @@
       <c r="Q66" s="92">
         <v>0.67</v>
       </c>
-      <c r="R66" s="11">
+      <c r="R66" s="92">
         <v>36.28</v>
       </c>
-      <c r="S66" s="11">
+      <c r="S66">
+        <v>72.3</v>
+      </c>
+      <c r="T66" s="11">
         <v>9105.6560000000009</v>
       </c>
-      <c r="T66" s="11">
+      <c r="U66" s="11">
         <v>24271.021387500001</v>
       </c>
-    </row>
-    <row r="67" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A67" s="89" t="s">
+      <c r="V66" s="11">
+        <v>115.18</v>
+      </c>
+    </row>
+    <row r="67" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A67" s="96" t="s">
         <v>915</v>
       </c>
       <c r="B67" s="89">
@@ -10805,18 +11081,24 @@
       <c r="Q67" s="92">
         <v>0.73</v>
       </c>
-      <c r="R67" s="11">
+      <c r="R67" s="92">
         <v>41.53</v>
       </c>
-      <c r="S67" s="11">
+      <c r="S67">
+        <v>78.099999999999994</v>
+      </c>
+      <c r="T67" s="11">
         <v>9839.9699999999993</v>
       </c>
-      <c r="T67" s="11">
+      <c r="U67" s="11">
         <v>26062.270152727269</v>
       </c>
-    </row>
-    <row r="68" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A68" s="88" t="s">
+      <c r="V67" s="11">
+        <v>115.89</v>
+      </c>
+    </row>
+    <row r="68" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A68" s="95" t="s">
         <v>916</v>
       </c>
       <c r="B68" s="88">
@@ -10867,18 +11149,24 @@
       <c r="Q68" s="92">
         <v>0.62</v>
       </c>
-      <c r="R68" s="11">
+      <c r="R68" s="92">
         <v>40.76</v>
       </c>
-      <c r="S68" s="11">
+      <c r="S68">
+        <v>72.5</v>
+      </c>
+      <c r="T68" s="11">
         <v>10499.862999999999</v>
       </c>
-      <c r="T68" s="11">
+      <c r="U68" s="11">
         <v>26385.830877272729</v>
       </c>
-    </row>
-    <row r="69" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A69" s="89" t="s">
+      <c r="V68" s="11">
+        <v>115.07</v>
+      </c>
+    </row>
+    <row r="69" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A69" s="96" t="s">
         <v>917</v>
       </c>
       <c r="B69" s="89">
@@ -10929,18 +11217,24 @@
       <c r="Q69" s="92">
         <v>0.65</v>
       </c>
-      <c r="R69" s="11">
+      <c r="R69" s="92">
         <v>44.71</v>
       </c>
-      <c r="S69" s="11">
+      <c r="S69">
+        <v>74.099999999999994</v>
+      </c>
+      <c r="T69" s="11">
         <v>11212.29</v>
       </c>
-      <c r="T69" s="11">
+      <c r="U69" s="11">
         <v>27821.367279999999</v>
       </c>
-    </row>
-    <row r="70" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A70" s="88" t="s">
+      <c r="V69" s="11">
+        <v>113.29</v>
+      </c>
+    </row>
+    <row r="70" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A70" s="95" t="s">
         <v>918</v>
       </c>
       <c r="B70" s="88">
@@ -10991,18 +11285,24 @@
       <c r="Q70" s="92">
         <v>0.68</v>
       </c>
-      <c r="R70" s="11">
+      <c r="R70" s="92">
         <v>38.450000000000003</v>
       </c>
-      <c r="S70" s="11">
+      <c r="S70">
+        <v>80.400000000000006</v>
+      </c>
+      <c r="T70" s="11">
         <v>11088.74</v>
       </c>
-      <c r="T70" s="11">
+      <c r="U70" s="11">
         <v>27733.396392857139</v>
       </c>
-    </row>
-    <row r="71" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A71" s="89" t="s">
+      <c r="V70" s="11">
+        <v>110.09</v>
+      </c>
+    </row>
+    <row r="71" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A71" s="96" t="s">
         <v>919</v>
       </c>
       <c r="B71" s="89">
@@ -11053,18 +11353,24 @@
       <c r="Q71" s="92">
         <v>0.79</v>
       </c>
-      <c r="R71" s="11">
+      <c r="R71" s="92">
         <v>40.380000000000003</v>
       </c>
-      <c r="S71" s="11">
+      <c r="S71">
+        <v>81.8</v>
+      </c>
+      <c r="T71" s="11">
         <v>11435.293</v>
       </c>
-      <c r="T71" s="11">
+      <c r="U71" s="11">
         <v>28005.105025909092</v>
       </c>
-    </row>
-    <row r="72" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A72" s="88" t="s">
+      <c r="V71" s="11">
+        <v>106.16</v>
+      </c>
+    </row>
+    <row r="72" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A72" s="95" t="s">
         <v>920</v>
       </c>
       <c r="B72" s="88">
@@ -11115,18 +11421,24 @@
       <c r="Q72" s="92">
         <v>0.87</v>
       </c>
-      <c r="R72" s="11">
+      <c r="R72" s="92">
         <v>40.869999999999997</v>
       </c>
-      <c r="S72" s="11">
+      <c r="S72">
+        <v>76.900000000000006</v>
+      </c>
+      <c r="T72" s="11">
         <v>11794.516</v>
       </c>
-      <c r="T72" s="11">
+      <c r="U72" s="11">
         <v>29124.036620999999</v>
       </c>
-    </row>
-    <row r="73" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A73" s="89" t="s">
+      <c r="V72" s="11">
+        <v>105.7</v>
+      </c>
+    </row>
+    <row r="73" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A73" s="96" t="s">
         <v>921</v>
       </c>
       <c r="B73" s="89">
@@ -11177,18 +11489,24 @@
       <c r="Q73" s="92">
         <v>0.93</v>
       </c>
-      <c r="R73" s="11">
+      <c r="R73" s="92">
         <v>39.76</v>
       </c>
-      <c r="S73" s="11">
+      <c r="S73">
+        <v>80.7</v>
+      </c>
+      <c r="T73" s="11">
         <v>12619.050999999999</v>
       </c>
-      <c r="T73" s="11">
+      <c r="U73" s="11">
         <v>30148.579900909092</v>
       </c>
-    </row>
-    <row r="74" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A74" s="88" t="s">
+      <c r="V73" s="11">
+        <v>107.58</v>
+      </c>
+    </row>
+    <row r="74" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A74" s="95" t="s">
         <v>922</v>
       </c>
       <c r="B74" s="88">
@@ -11239,18 +11557,24 @@
       <c r="Q74" s="92">
         <v>1.08</v>
       </c>
-      <c r="R74" s="11">
+      <c r="R74" s="92">
         <v>36.909999999999997</v>
       </c>
-      <c r="S74" s="11">
+      <c r="S74">
+        <v>79</v>
+      </c>
+      <c r="T74" s="11">
         <v>13186.606</v>
       </c>
-      <c r="T74" s="11">
+      <c r="U74" s="11">
         <v>30821.35259052632</v>
       </c>
-    </row>
-    <row r="75" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A75" s="89" t="s">
+      <c r="V74" s="11">
+        <v>109.73</v>
+      </c>
+    </row>
+    <row r="75" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A75" s="96" t="s">
         <v>923</v>
       </c>
       <c r="B75" s="89">
@@ -11301,18 +11625,24 @@
       <c r="Q75" s="92">
         <v>1.26</v>
       </c>
-      <c r="R75" s="11">
+      <c r="R75" s="92">
         <v>38.119999999999997</v>
       </c>
-      <c r="S75" s="11">
+      <c r="S75">
+        <v>76.8</v>
+      </c>
+      <c r="T75" s="11">
         <v>13737.405000000001</v>
       </c>
-      <c r="T75" s="11">
+      <c r="U75" s="11">
         <v>31283.909848421052</v>
       </c>
-    </row>
-    <row r="76" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A76" s="88" t="s">
+      <c r="V75" s="11">
+        <v>112.95</v>
+      </c>
+    </row>
+    <row r="76" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A76" s="95" t="s">
         <v>924</v>
       </c>
       <c r="B76" s="88">
@@ -11363,18 +11693,24 @@
       <c r="Q76" s="92">
         <v>1.61</v>
       </c>
-      <c r="R76" s="11">
+      <c r="R76" s="92">
         <v>36.76</v>
       </c>
-      <c r="S76" s="11">
+      <c r="S76">
+        <v>84.9</v>
+      </c>
+      <c r="T76" s="11">
         <v>13168.811</v>
       </c>
-      <c r="T76" s="11">
+      <c r="U76" s="11">
         <v>32373.291100434781</v>
       </c>
-    </row>
-    <row r="77" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A77" s="89" t="s">
+      <c r="V76" s="11">
+        <v>115.19</v>
+      </c>
+    </row>
+    <row r="77" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A77" s="96" t="s">
         <v>925</v>
       </c>
       <c r="B77" s="89">
@@ -11425,18 +11761,24 @@
       <c r="Q77" s="92">
         <v>1.64</v>
       </c>
-      <c r="R77" s="11">
+      <c r="R77" s="92">
         <v>37.6</v>
       </c>
-      <c r="S77" s="11">
+      <c r="S77">
+        <v>88.3</v>
+      </c>
+      <c r="T77" s="11">
         <v>13900.438</v>
       </c>
-      <c r="T77" s="11">
+      <c r="U77" s="11">
         <v>33803.286087142857</v>
       </c>
-    </row>
-    <row r="78" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A78" s="88" t="s">
+      <c r="V77" s="11">
+        <v>116.11</v>
+      </c>
+    </row>
+    <row r="78" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A78" s="95" t="s">
         <v>926</v>
       </c>
       <c r="B78" s="88">
@@ -11487,18 +11829,24 @@
       <c r="Q78" s="92">
         <v>1.62</v>
       </c>
-      <c r="R78" s="11">
+      <c r="R78" s="92">
         <v>35.79</v>
       </c>
-      <c r="S78" s="11">
+      <c r="S78">
+        <v>82.9</v>
+      </c>
+      <c r="T78" s="11">
         <v>13520.228999999999</v>
       </c>
-      <c r="T78" s="11">
+      <c r="U78" s="11">
         <v>34270.308594499998</v>
       </c>
-    </row>
-    <row r="79" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A79" s="89" t="s">
+      <c r="V78" s="11">
+        <v>117.86</v>
+      </c>
+    </row>
+    <row r="79" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A79" s="96" t="s">
         <v>927</v>
       </c>
       <c r="B79" s="89">
@@ -11549,18 +11897,24 @@
       <c r="Q79" s="92">
         <v>1.52</v>
       </c>
-      <c r="R79" s="11">
+      <c r="R79" s="92">
         <v>35.630000000000003</v>
       </c>
-      <c r="S79" s="11">
+      <c r="S79">
+        <v>85.5</v>
+      </c>
+      <c r="T79" s="11">
         <v>14097.169</v>
       </c>
-      <c r="T79" s="11">
+      <c r="U79" s="11">
         <v>34289.906783181817</v>
       </c>
-    </row>
-    <row r="80" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A80" s="88" t="s">
+      <c r="V79" s="11">
+        <v>118.97</v>
+      </c>
+    </row>
+    <row r="80" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A80" s="95" t="s">
         <v>928</v>
       </c>
       <c r="B80" s="88">
@@ -11611,18 +11965,24 @@
       <c r="Q80" s="92">
         <v>1.32</v>
       </c>
-      <c r="R80" s="11">
+      <c r="R80" s="92">
         <v>39.229999999999997</v>
       </c>
-      <c r="S80" s="11">
+      <c r="S80">
+        <v>81.2</v>
+      </c>
+      <c r="T80" s="11">
         <v>14639.073</v>
       </c>
-      <c r="T80" s="11">
+      <c r="U80" s="11">
         <v>34798.804314761903</v>
       </c>
-    </row>
-    <row r="81" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A81" s="89" t="s">
+      <c r="V80" s="11">
+        <v>119.52</v>
+      </c>
+    </row>
+    <row r="81" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A81" s="96" t="s">
         <v>929</v>
       </c>
       <c r="B81" s="89">
@@ -11673,18 +12033,24 @@
       <c r="Q81" s="92">
         <v>1.28</v>
       </c>
-      <c r="R81" s="11">
+      <c r="R81" s="92">
         <v>37.76</v>
       </c>
-      <c r="S81" s="11">
+      <c r="S81">
+        <v>70.3</v>
+      </c>
+      <c r="T81" s="11">
         <v>14856.518</v>
       </c>
-      <c r="T81" s="11">
+      <c r="U81" s="11">
         <v>35243.965909999999</v>
       </c>
-    </row>
-    <row r="82" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A82" s="88" t="s">
+      <c r="V81" s="11">
+        <v>121.59</v>
+      </c>
+    </row>
+    <row r="82" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A82" s="95" t="s">
         <v>930</v>
       </c>
       <c r="B82" s="88">
@@ -11735,18 +12101,24 @@
       <c r="Q82" s="92">
         <v>1.37</v>
       </c>
-      <c r="R82" s="11">
+      <c r="R82" s="92">
         <v>38.47</v>
       </c>
-      <c r="S82" s="11">
+      <c r="S82">
+        <v>72.8</v>
+      </c>
+      <c r="T82" s="11">
         <v>15023.539000000001</v>
       </c>
-      <c r="T82" s="11">
+      <c r="U82" s="11">
         <v>34688.421316666667</v>
       </c>
-    </row>
-    <row r="83" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A83" s="89" t="s">
+      <c r="V82" s="11">
+        <v>122.51</v>
+      </c>
+    </row>
+    <row r="83" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A83" s="96" t="s">
         <v>931</v>
       </c>
       <c r="B83" s="89">
@@ -11797,18 +12169,24 @@
       <c r="Q83" s="92">
         <v>1.58</v>
       </c>
-      <c r="R83" s="11">
+      <c r="R83" s="92">
         <v>40.18</v>
       </c>
-      <c r="S83" s="11">
+      <c r="S83">
+        <v>71.7</v>
+      </c>
+      <c r="T83" s="11">
         <v>14879.012000000001</v>
       </c>
-      <c r="T83" s="11">
+      <c r="U83" s="11">
         <v>35055.517857619037</v>
       </c>
-    </row>
-    <row r="84" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A84" s="88" t="s">
+      <c r="V83" s="11">
+        <v>121.85</v>
+      </c>
+    </row>
+    <row r="84" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A84" s="95" t="s">
         <v>932</v>
       </c>
       <c r="B84" s="88">
@@ -11859,18 +12237,24 @@
       <c r="Q84" s="92">
         <v>1.56</v>
       </c>
-      <c r="R84" s="11">
+      <c r="R84" s="92">
         <v>40.020000000000003</v>
       </c>
-      <c r="S84" s="11">
+      <c r="S84">
+        <v>67.400000000000006</v>
+      </c>
+      <c r="T84" s="11">
         <v>15814.933000000001</v>
       </c>
-      <c r="T84" s="11">
+      <c r="U84" s="11">
         <v>35848.570685238097</v>
       </c>
-    </row>
-    <row r="85" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A85" s="89" t="s">
+      <c r="V84" s="11">
+        <v>121.92</v>
+      </c>
+    </row>
+    <row r="85" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A85" s="96" t="s">
         <v>933</v>
       </c>
       <c r="B85" s="89">
@@ -11921,18 +12305,24 @@
       <c r="Q85" s="92">
         <v>1.47</v>
       </c>
-      <c r="R85" s="11">
+      <c r="R85" s="92">
         <v>38.74</v>
       </c>
-      <c r="S85" s="11">
+      <c r="S85">
+        <v>70.599999999999994</v>
+      </c>
+      <c r="T85" s="11">
         <v>15474.432000000001</v>
       </c>
-      <c r="T85" s="11">
+      <c r="U85" s="11">
         <v>35641.333808636373</v>
       </c>
-    </row>
-    <row r="86" spans="1:20" s="11" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
-      <c r="A86" s="88" t="s">
+      <c r="V85" s="11">
+        <v>121.08</v>
+      </c>
+    </row>
+    <row r="86" spans="1:22" s="11" customFormat="1" ht="14.5" x14ac:dyDescent="0.35">
+      <c r="A86" s="95" t="s">
         <v>934</v>
       </c>
       <c r="B86" s="88">
@@ -11983,18 +12373,24 @@
       <c r="Q86" s="92">
         <v>1.76</v>
       </c>
-      <c r="R86" s="11">
+      <c r="R86" s="92">
         <v>41</v>
       </c>
-      <c r="S86" s="11">
+      <c r="S86">
+        <v>67.2</v>
+      </c>
+      <c r="T86" s="11">
         <v>14531.378000000001</v>
       </c>
-      <c r="T86" s="11">
+      <c r="U86" s="11">
         <v>35456.144726500002</v>
       </c>
-    </row>
-    <row r="87" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A87" s="89" t="s">
+      <c r="V86" s="11">
+        <v>119.08</v>
+      </c>
+    </row>
+    <row r="87" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A87" s="96" t="s">
         <v>935</v>
       </c>
       <c r="B87" s="89">
@@ -12045,18 +12441,24 @@
       <c r="Q87" s="92">
         <v>1.93</v>
       </c>
-      <c r="R87" s="11">
+      <c r="R87" s="92">
         <v>40.71</v>
       </c>
-      <c r="S87" s="11">
+      <c r="S87">
+        <v>62.8</v>
+      </c>
+      <c r="T87" s="11">
         <v>13898.727999999999</v>
       </c>
-      <c r="T87" s="11">
+      <c r="U87" s="11">
         <v>34648.480263684207</v>
       </c>
-    </row>
-    <row r="88" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A88" s="88" t="s">
+      <c r="V87" s="11">
+        <v>118.51</v>
+      </c>
+    </row>
+    <row r="88" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A88" s="95" t="s">
         <v>936</v>
       </c>
       <c r="B88" s="88">
@@ -12107,18 +12509,24 @@
       <c r="Q88" s="92">
         <v>2.13</v>
       </c>
-      <c r="R88" s="11">
+      <c r="R88" s="92">
         <v>37.96</v>
       </c>
-      <c r="S88" s="11">
+      <c r="S88">
+        <v>59.4</v>
+      </c>
+      <c r="T88" s="11">
         <v>13623.263000000001</v>
       </c>
-      <c r="T88" s="11">
+      <c r="U88" s="11">
         <v>34029.740659565221</v>
       </c>
-    </row>
-    <row r="89" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A89" s="89" t="s">
+      <c r="V88" s="11">
+        <v>118.17</v>
+      </c>
+    </row>
+    <row r="89" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A89" s="96" t="s">
         <v>937</v>
       </c>
       <c r="B89" s="89">
@@ -12169,18 +12577,24 @@
       <c r="Q89" s="92">
         <v>2.75</v>
       </c>
-      <c r="R89" s="11">
+      <c r="R89" s="92">
         <v>40.97</v>
       </c>
-      <c r="S89" s="11">
+      <c r="S89">
+        <v>65.2</v>
+      </c>
+      <c r="T89" s="11">
         <v>13394.163</v>
       </c>
-      <c r="T89" s="11">
+      <c r="U89" s="11">
         <v>34314.990040500001</v>
       </c>
-    </row>
-    <row r="90" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A90" s="88" t="s">
+      <c r="V89" s="11">
+        <v>115.85</v>
+      </c>
+    </row>
+    <row r="90" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A90" s="95" t="s">
         <v>938</v>
       </c>
       <c r="B90" s="88">
@@ -12231,18 +12645,24 @@
       <c r="Q90" s="92">
         <v>2.9</v>
       </c>
-      <c r="R90" s="11">
+      <c r="R90" s="92">
         <v>35.58</v>
       </c>
-      <c r="S90" s="11">
+      <c r="S90">
+        <v>58.4</v>
+      </c>
+      <c r="T90" s="11">
         <v>11829.73</v>
       </c>
-      <c r="T90" s="11">
+      <c r="U90" s="11">
         <v>32379.46279666667</v>
       </c>
-    </row>
-    <row r="91" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A91" s="89" t="s">
+      <c r="V90" s="11">
+        <v>113.3</v>
+      </c>
+    </row>
+    <row r="91" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A91" s="96" t="s">
         <v>939</v>
       </c>
       <c r="B91" s="89">
@@ -12293,18 +12713,24 @@
       <c r="Q91" s="92">
         <v>3.14</v>
       </c>
-      <c r="R91" s="11">
+      <c r="R91" s="92">
         <v>40.380000000000003</v>
       </c>
-      <c r="S91" s="11">
+      <c r="S91">
+        <v>50</v>
+      </c>
+      <c r="T91" s="11">
         <v>11418.919</v>
       </c>
-      <c r="T91" s="11">
+      <c r="U91" s="11">
         <v>31446.712798571429</v>
       </c>
-    </row>
-    <row r="92" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A92" s="88" t="s">
+      <c r="V91" s="11">
+        <v>111.96</v>
+      </c>
+    </row>
+    <row r="92" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A92" s="95" t="s">
         <v>940</v>
       </c>
       <c r="B92" s="88">
@@ -12355,18 +12781,24 @@
       <c r="Q92" s="92">
         <v>2.9</v>
       </c>
-      <c r="R92" s="11">
+      <c r="R92" s="92">
         <v>38.39</v>
       </c>
-      <c r="S92" s="11">
+      <c r="S92">
+        <v>51.5</v>
+      </c>
+      <c r="T92" s="11">
         <v>11622.632</v>
       </c>
-      <c r="T92" s="11">
+      <c r="U92" s="11">
         <v>31535.323339499999</v>
       </c>
-    </row>
-    <row r="93" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A93" s="89" t="s">
+      <c r="V92" s="11">
+        <v>110.53</v>
+      </c>
+    </row>
+    <row r="93" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A93" s="96" t="s">
         <v>941</v>
       </c>
       <c r="B93" s="89">
@@ -12417,18 +12849,24 @@
       <c r="Q93" s="92">
         <v>2.9</v>
       </c>
-      <c r="R93" s="11">
+      <c r="R93" s="92">
         <v>38.950000000000003</v>
       </c>
-      <c r="S93" s="11">
+      <c r="S93">
+        <v>58.2</v>
+      </c>
+      <c r="T93" s="11">
         <v>12570.26</v>
       </c>
-      <c r="T93" s="11">
+      <c r="U93" s="11">
         <v>33009.564877826087</v>
       </c>
-    </row>
-    <row r="94" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A94" s="88" t="s">
+      <c r="V93" s="11">
+        <v>109.83</v>
+      </c>
+    </row>
+    <row r="94" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A94" s="95" t="s">
         <v>942</v>
       </c>
       <c r="B94" s="88">
@@ -12479,18 +12917,24 @@
       <c r="Q94" s="92">
         <v>3.52</v>
       </c>
-      <c r="R94" s="11">
+      <c r="R94" s="92">
         <v>36.21</v>
       </c>
-      <c r="S94" s="11">
+      <c r="S94">
+        <v>58.6</v>
+      </c>
+      <c r="T94" s="11">
         <v>11402.85</v>
       </c>
-      <c r="T94" s="11">
+      <c r="U94" s="11">
         <v>30649.559523809519</v>
       </c>
-    </row>
-    <row r="95" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A95" s="89" t="s">
+      <c r="V94" s="11">
+        <v>109.94</v>
+      </c>
+    </row>
+    <row r="95" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A95" s="96" t="s">
         <v>943</v>
       </c>
       <c r="B95" s="89">
@@ -12541,18 +12985,24 @@
       <c r="Q95" s="92">
         <v>3.98</v>
       </c>
-      <c r="R95" s="11">
+      <c r="R95" s="92">
         <v>37.46</v>
       </c>
-      <c r="S95" s="11">
+      <c r="S95">
+        <v>59.9</v>
+      </c>
+      <c r="T95" s="11">
         <v>10801.494000000001</v>
       </c>
-      <c r="T95" s="11">
+      <c r="U95" s="11">
         <v>30570.68377952381</v>
       </c>
-    </row>
-    <row r="96" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A96" s="88" t="s">
+      <c r="V95" s="11">
+        <v>108.27</v>
+      </c>
+    </row>
+    <row r="96" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A96" s="95" t="s">
         <v>944</v>
       </c>
       <c r="B96" s="88">
@@ -12603,18 +13053,24 @@
       <c r="Q96" s="92">
         <v>3.89</v>
       </c>
-      <c r="R96" s="11">
+      <c r="R96" s="92">
         <v>34.049999999999997</v>
       </c>
-      <c r="S96" s="11">
+      <c r="S96">
+        <v>56.7</v>
+      </c>
+      <c r="T96" s="11">
         <v>10973.638000000001</v>
       </c>
-      <c r="T96" s="11">
+      <c r="U96" s="11">
         <v>33417.958240952379</v>
       </c>
-    </row>
-    <row r="97" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A97" s="89" t="s">
+      <c r="V96" s="11">
+        <v>104.47</v>
+      </c>
+    </row>
+    <row r="97" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A97" s="96" t="s">
         <v>945</v>
       </c>
       <c r="B97" s="89">
@@ -12665,18 +13121,24 @@
       <c r="Q97" s="92">
         <v>3.62</v>
       </c>
-      <c r="R97" s="11">
+      <c r="R97" s="92">
         <v>39.229999999999997</v>
       </c>
-      <c r="S97" s="11">
+      <c r="S97">
+        <v>59.8</v>
+      </c>
+      <c r="T97" s="11">
         <v>10838.995999999999</v>
       </c>
-      <c r="T97" s="11">
+      <c r="U97" s="11">
         <v>33482.257254761913</v>
       </c>
-    </row>
-    <row r="98" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A98" s="88" t="s">
+      <c r="V97" s="11">
+        <v>101.89</v>
+      </c>
+    </row>
+    <row r="98" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A98" s="95" t="s">
         <v>946</v>
       </c>
       <c r="B98" s="88">
@@ -12727,18 +13189,24 @@
       <c r="Q98" s="92">
         <v>3.53</v>
       </c>
-      <c r="R98" s="11">
+      <c r="R98" s="92">
         <v>38.770000000000003</v>
       </c>
-      <c r="S98" s="11">
+      <c r="S98">
+        <v>64.900000000000006</v>
+      </c>
+      <c r="T98" s="11">
         <v>11013.991</v>
       </c>
-      <c r="T98" s="11">
+      <c r="U98" s="11">
         <v>33656.000195499997</v>
       </c>
-    </row>
-    <row r="99" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A99" s="89" t="s">
+      <c r="V98" s="11">
+        <v>99.41</v>
+      </c>
+    </row>
+    <row r="99" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A99" s="96" t="s">
         <v>947</v>
       </c>
       <c r="B99" s="89">
@@ -12789,18 +13257,24 @@
       <c r="Q99" s="92">
         <v>3.75</v>
       </c>
-      <c r="R99" s="11">
+      <c r="R99" s="92">
         <v>35.78</v>
       </c>
-      <c r="S99" s="11">
+      <c r="S99">
+        <v>66.900000000000006</v>
+      </c>
+      <c r="T99" s="11">
         <v>11785.074000000001</v>
       </c>
-      <c r="T99" s="11">
+      <c r="U99" s="11">
         <v>33648.256785263147</v>
       </c>
-    </row>
-    <row r="100" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A100" s="88" t="s">
+      <c r="V99" s="11">
+        <v>93.87</v>
+      </c>
+    </row>
+    <row r="100" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A100" s="95" t="s">
         <v>948</v>
       </c>
       <c r="B100" s="88">
@@ -12851,18 +13325,24 @@
       <c r="Q100" s="92">
         <v>3.66</v>
       </c>
-      <c r="R100" s="11">
+      <c r="R100" s="92">
         <v>39.729999999999997</v>
       </c>
-      <c r="S100" s="11">
+      <c r="S100">
+        <v>62</v>
+      </c>
+      <c r="T100" s="11">
         <v>11637.092000000001</v>
       </c>
-      <c r="T100" s="11">
+      <c r="U100" s="11">
         <v>32483.47826217391</v>
       </c>
-    </row>
-    <row r="101" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A101" s="89" t="s">
+      <c r="V100" s="11">
+        <v>89.18</v>
+      </c>
+    </row>
+    <row r="101" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A101" s="96" t="s">
         <v>949</v>
       </c>
       <c r="B101" s="89">
@@ -12913,18 +13393,24 @@
       <c r="Q101" s="92">
         <v>3.46</v>
       </c>
-      <c r="R101" s="11">
+      <c r="R101" s="92">
         <v>36.880000000000003</v>
       </c>
-      <c r="S101" s="11">
+      <c r="S101">
+        <v>63.7</v>
+      </c>
+      <c r="T101" s="11">
         <v>12073.465</v>
       </c>
-      <c r="T101" s="11">
+      <c r="U101" s="11">
         <v>33731.280223157897</v>
       </c>
-    </row>
-    <row r="102" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A102" s="88" t="s">
+      <c r="V101" s="11">
+        <v>86.83</v>
+      </c>
+    </row>
+    <row r="102" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A102" s="95" t="s">
         <v>950</v>
       </c>
       <c r="B102" s="88">
@@ -12975,18 +13461,24 @@
       <c r="Q102" s="92">
         <v>3.57</v>
       </c>
-      <c r="R102" s="11">
+      <c r="R102" s="92">
         <v>38.53</v>
       </c>
-      <c r="S102" s="11">
+      <c r="S102">
+        <v>59</v>
+      </c>
+      <c r="T102" s="11">
         <v>12446.53</v>
       </c>
-      <c r="T102" s="11">
+      <c r="U102" s="11">
         <v>33316.802291363638</v>
       </c>
-    </row>
-    <row r="103" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A103" s="89" t="s">
+      <c r="V102" s="11">
+        <v>84.52</v>
+      </c>
+    </row>
+    <row r="103" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A103" s="96" t="s">
         <v>951</v>
       </c>
       <c r="B103" s="89">
@@ -13037,18 +13529,24 @@
       <c r="Q103" s="92">
         <v>3.75</v>
       </c>
-      <c r="R103" s="11">
+      <c r="R103" s="92">
         <v>42.25</v>
       </c>
-      <c r="S103" s="11">
+      <c r="S103">
+        <v>64.2</v>
+      </c>
+      <c r="T103" s="11">
         <v>13463.778</v>
       </c>
-      <c r="T103" s="11">
+      <c r="U103" s="11">
         <v>33904.976377142862</v>
       </c>
-    </row>
-    <row r="104" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A104" s="88" t="s">
+      <c r="V103" s="11">
+        <v>84.24</v>
+      </c>
+    </row>
+    <row r="104" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A104" s="95" t="s">
         <v>952</v>
       </c>
       <c r="B104" s="88">
@@ -13099,18 +13597,24 @@
       <c r="Q104" s="92">
         <v>3.9</v>
       </c>
-      <c r="R104" s="11">
+      <c r="R104" s="92">
         <v>43.39</v>
       </c>
-      <c r="S104" s="11">
+      <c r="S104">
+        <v>71.5</v>
+      </c>
+      <c r="T104" s="11">
         <v>14033.091</v>
       </c>
-      <c r="T104" s="11">
+      <c r="U104" s="11">
         <v>34777.200196500002</v>
       </c>
-    </row>
-    <row r="105" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A105" s="89" t="s">
+      <c r="V104" s="11">
+        <v>87.01</v>
+      </c>
+    </row>
+    <row r="105" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A105" s="96" t="s">
         <v>953</v>
       </c>
       <c r="B105" s="89">
@@ -13161,18 +13665,24 @@
       <c r="Q105" s="92">
         <v>4.17</v>
       </c>
-      <c r="R105" s="11">
+      <c r="R105" s="92">
         <v>46.13</v>
       </c>
-      <c r="S105" s="11">
+      <c r="S105">
+        <v>69.400000000000006</v>
+      </c>
+      <c r="T105" s="11">
         <v>13739.496999999999</v>
       </c>
-      <c r="T105" s="11">
+      <c r="U105" s="11">
         <v>34880.656592173909</v>
       </c>
-    </row>
-    <row r="106" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A106" s="88" t="s">
+      <c r="V105" s="11">
+        <v>90.6</v>
+      </c>
+    </row>
+    <row r="106" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A106" s="95" t="s">
         <v>954</v>
       </c>
       <c r="B106" s="88">
@@ -13223,18 +13733,24 @@
       <c r="Q106" s="92">
         <v>4.38</v>
       </c>
-      <c r="R106" s="11">
+      <c r="R106" s="92">
         <v>42.87</v>
       </c>
-      <c r="S106" s="11">
+      <c r="S106">
+        <v>67.8</v>
+      </c>
+      <c r="T106" s="11">
         <v>13585.842000000001</v>
       </c>
-      <c r="T106" s="11">
+      <c r="U106" s="11">
         <v>34318.890821000001</v>
       </c>
-    </row>
-    <row r="107" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A107" s="89" t="s">
+      <c r="V106" s="11">
+        <v>94.32</v>
+      </c>
+    </row>
+    <row r="107" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A107" s="96" t="s">
         <v>955</v>
       </c>
       <c r="B107" s="89">
@@ -13285,18 +13801,24 @@
       <c r="Q107" s="92">
         <v>4.8</v>
       </c>
-      <c r="R107" s="11">
+      <c r="R107" s="92">
         <v>44.13</v>
       </c>
-      <c r="S107" s="11">
+      <c r="S107">
+        <v>63.8</v>
+      </c>
+      <c r="T107" s="11">
         <v>13199.428</v>
       </c>
-      <c r="T107" s="11">
+      <c r="U107" s="11">
         <v>33319.492720909089</v>
       </c>
-    </row>
-    <row r="108" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A108" s="88" t="s">
+      <c r="V107" s="11">
+        <v>96.89</v>
+      </c>
+    </row>
+    <row r="108" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A108" s="95" t="s">
         <v>956</v>
       </c>
       <c r="B108" s="88">
@@ -13347,18 +13869,24 @@
       <c r="Q108" s="92">
         <v>4.5</v>
       </c>
-      <c r="R108" s="11">
+      <c r="R108" s="92">
         <v>46.77</v>
       </c>
-      <c r="S108" s="11">
+      <c r="S108">
+        <v>61.3</v>
+      </c>
+      <c r="T108" s="11">
         <v>13913.16</v>
       </c>
-      <c r="T108" s="11">
+      <c r="U108" s="11">
         <v>34704.502419047618</v>
       </c>
-    </row>
-    <row r="109" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A109" s="89" t="s">
+      <c r="V108" s="11">
+        <v>98.32</v>
+      </c>
+    </row>
+    <row r="109" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A109" s="96" t="s">
         <v>957</v>
       </c>
       <c r="B109" s="89">
@@ -13409,18 +13937,24 @@
       <c r="Q109" s="92">
         <v>4.0199999999999996</v>
       </c>
-      <c r="R109" s="11">
+      <c r="R109" s="92">
         <v>40.44</v>
       </c>
-      <c r="S109" s="11">
+      <c r="S109">
+        <v>69.7</v>
+      </c>
+      <c r="T109" s="11">
         <v>14690.493</v>
       </c>
-      <c r="T109" s="11">
+      <c r="U109" s="11">
         <v>36947.9275395</v>
       </c>
-    </row>
-    <row r="110" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A110" s="88" t="s">
+      <c r="V109" s="11">
+        <v>100.71</v>
+      </c>
+    </row>
+    <row r="110" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A110" s="95" t="s">
         <v>958</v>
       </c>
       <c r="B110" s="88">
@@ -13471,18 +14005,24 @@
       <c r="Q110" s="92">
         <v>4.0599999999999996</v>
       </c>
-      <c r="R110" s="11">
+      <c r="R110" s="92">
         <v>32.74</v>
       </c>
-      <c r="S110" s="11">
+      <c r="S110">
+        <v>79</v>
+      </c>
+      <c r="T110" s="11">
         <v>15081.388000000001</v>
       </c>
-      <c r="T110" s="11">
+      <c r="U110" s="11">
         <v>37763.9548</v>
       </c>
-    </row>
-    <row r="111" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A111" s="89" t="s">
+      <c r="V110" s="11">
+        <v>104.44</v>
+      </c>
+    </row>
+    <row r="111" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A111" s="96" t="s">
         <v>959</v>
       </c>
       <c r="B111" s="89">
@@ -13533,18 +14073,24 @@
       <c r="Q111" s="92">
         <v>4.21</v>
       </c>
-      <c r="R111" s="11">
+      <c r="R111" s="92">
         <v>33.76</v>
       </c>
-      <c r="S111" s="11">
+      <c r="S111">
+        <v>76.900000000000006</v>
+      </c>
+      <c r="T111" s="11">
         <v>15808.934999999999</v>
       </c>
-      <c r="T111" s="11">
+      <c r="U111" s="11">
         <v>38720.517970000001</v>
       </c>
-    </row>
-    <row r="112" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A112" s="88" t="s">
+      <c r="V111" s="11">
+        <v>107.9</v>
+      </c>
+    </row>
+    <row r="112" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A112" s="95" t="s">
         <v>960</v>
       </c>
       <c r="B112" s="88">
@@ -13595,18 +14141,24 @@
       <c r="Q112" s="92">
         <v>4.21</v>
       </c>
-      <c r="R112" s="11">
+      <c r="R112" s="92">
         <v>36.43</v>
       </c>
-      <c r="S112" s="11">
+      <c r="S112">
+        <v>79.400000000000006</v>
+      </c>
+      <c r="T112" s="11">
         <v>16216.296</v>
       </c>
-      <c r="T112" s="11">
+      <c r="U112" s="11">
         <v>39105.519923499996</v>
       </c>
-    </row>
-    <row r="113" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A113" s="89" t="s">
+      <c r="V112" s="11">
+        <v>112.9</v>
+      </c>
+    </row>
+    <row r="113" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A113" s="96" t="s">
         <v>961</v>
       </c>
       <c r="B113" s="89">
@@ -13657,18 +14209,24 @@
       <c r="Q113" s="92">
         <v>4.54</v>
       </c>
-      <c r="R113" s="11">
+      <c r="R113" s="92">
         <v>38.450000000000003</v>
       </c>
-      <c r="S113" s="11">
+      <c r="S113">
+        <v>77.2</v>
+      </c>
+      <c r="T113" s="11">
         <v>15950.864</v>
       </c>
-      <c r="T113" s="11">
+      <c r="U113" s="11">
         <v>38401.217330909087</v>
       </c>
-    </row>
-    <row r="114" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A114" s="88" t="s">
+      <c r="V113" s="11">
+        <v>118.54</v>
+      </c>
+    </row>
+    <row r="114" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A114" s="95" t="s">
         <v>962</v>
       </c>
       <c r="B114" s="88">
@@ -13719,18 +14277,24 @@
       <c r="Q114" s="92">
         <v>4.4800000000000004</v>
       </c>
-      <c r="R114" s="11">
+      <c r="R114" s="92">
         <v>41.84</v>
       </c>
-      <c r="S114" s="11">
+      <c r="S114">
+        <v>69.099999999999994</v>
+      </c>
+      <c r="T114" s="11">
         <v>16536.316999999999</v>
       </c>
-      <c r="T114" s="11">
+      <c r="U114" s="11">
         <v>39129.390447727274</v>
       </c>
-    </row>
-    <row r="115" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A115" s="89" t="s">
+      <c r="V114" s="11">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="115" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A115" s="96" t="s">
         <v>963</v>
       </c>
       <c r="B115" s="89">
@@ -13781,18 +14345,24 @@
       <c r="Q115" s="92">
         <v>4.3099999999999996</v>
       </c>
-      <c r="R115" s="11">
+      <c r="R115" s="92">
         <v>35.96</v>
       </c>
-      <c r="S115" s="11">
+      <c r="S115">
+        <v>68.2</v>
+      </c>
+      <c r="T115" s="11">
         <v>17495.892</v>
       </c>
-      <c r="T115" s="11">
+      <c r="U115" s="11">
         <v>38903.730675789477</v>
       </c>
-    </row>
-    <row r="116" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A116" s="88" t="s">
+      <c r="V115" s="11">
+        <v>117.31</v>
+      </c>
+    </row>
+    <row r="116" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A116" s="95" t="s">
         <v>964</v>
       </c>
       <c r="B116" s="88">
@@ -13843,18 +14413,24 @@
       <c r="Q116" s="92">
         <v>4.25</v>
       </c>
-      <c r="R116" s="11">
+      <c r="R116" s="92">
         <v>36.31</v>
       </c>
-      <c r="S116" s="11">
+      <c r="S116">
+        <v>66.400000000000006</v>
+      </c>
+      <c r="T116" s="11">
         <v>17963.291000000001</v>
       </c>
-      <c r="T116" s="11">
+      <c r="U116" s="11">
         <v>40086.031604999996</v>
       </c>
-    </row>
-    <row r="117" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A117" s="89" t="s">
+      <c r="V116" s="11">
+        <v>113.3</v>
+      </c>
+    </row>
+    <row r="117" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A117" s="96" t="s">
         <v>965</v>
       </c>
       <c r="B117" s="89">
@@ -13905,18 +14481,24 @@
       <c r="Q117" s="92">
         <v>3.87</v>
       </c>
-      <c r="R117" s="11">
+      <c r="R117" s="92">
         <v>42.96</v>
       </c>
-      <c r="S117" s="11">
+      <c r="S117">
+        <v>67.900000000000006</v>
+      </c>
+      <c r="T117" s="11">
         <v>17268.269</v>
       </c>
-      <c r="T117" s="11">
+      <c r="U117" s="11">
         <v>40310.814454090912</v>
       </c>
-    </row>
-    <row r="118" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A118" s="88" t="s">
+      <c r="V117" s="11">
+        <v>110.75</v>
+      </c>
+    </row>
+    <row r="118" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A118" s="95" t="s">
         <v>966</v>
       </c>
       <c r="B118" s="88">
@@ -13967,18 +14549,24 @@
       <c r="Q118" s="92">
         <v>3.72</v>
       </c>
-      <c r="R118" s="11">
+      <c r="R118" s="92">
         <v>38.79</v>
       </c>
-      <c r="S118" s="11">
+      <c r="S118">
+        <v>70.099999999999994</v>
+      </c>
+      <c r="T118" s="11">
         <v>17599.23</v>
       </c>
-      <c r="T118" s="11">
+      <c r="U118" s="11">
         <v>41490.882813999997</v>
       </c>
-    </row>
-    <row r="119" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A119" s="89" t="s">
+      <c r="V118" s="11">
+        <v>111.43</v>
+      </c>
+    </row>
+    <row r="119" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A119" s="96" t="s">
         <v>967</v>
       </c>
       <c r="B119" s="89">
@@ -14029,18 +14617,24 @@
       <c r="Q119" s="92">
         <v>4.0999999999999996</v>
       </c>
-      <c r="R119" s="11">
+      <c r="R119" s="92">
         <v>39.46</v>
       </c>
-      <c r="S119" s="11">
+      <c r="S119">
+        <v>70.5</v>
+      </c>
+      <c r="T119" s="11">
         <v>18316.116000000002</v>
       </c>
-      <c r="T119" s="11">
+      <c r="U119" s="11">
         <v>42494.197350869566</v>
       </c>
-    </row>
-    <row r="120" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A120" s="88" t="s">
+      <c r="V119" s="11">
+        <v>113.07</v>
+      </c>
+    </row>
+    <row r="120" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A120" s="95" t="s">
         <v>968</v>
       </c>
       <c r="B120" s="88">
@@ -14091,18 +14685,24 @@
       <c r="Q120" s="92">
         <v>4.3600000000000003</v>
       </c>
-      <c r="R120" s="11">
+      <c r="R120" s="92">
         <v>44.42</v>
       </c>
-      <c r="S120" s="11">
+      <c r="S120">
+        <v>71.8</v>
+      </c>
+      <c r="T120" s="11">
         <v>18961.400000000001</v>
       </c>
-      <c r="T120" s="11">
+      <c r="U120" s="11">
         <v>43716.926953499998</v>
       </c>
-    </row>
-    <row r="121" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A121" s="89" t="s">
+      <c r="V120" s="11">
+        <v>114.67</v>
+      </c>
+    </row>
+    <row r="121" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A121" s="96" t="s">
         <v>969</v>
       </c>
       <c r="B121" s="89">
@@ -14153,18 +14753,24 @@
       <c r="Q121" s="92">
         <v>4.3899999999999997</v>
       </c>
-      <c r="R121" s="11">
+      <c r="R121" s="92">
         <v>42.17</v>
       </c>
-      <c r="S121" s="11">
+      <c r="S121">
+        <v>74</v>
+      </c>
+      <c r="T121" s="11">
         <v>19734.563999999998</v>
       </c>
-      <c r="T121" s="11">
+      <c r="U121" s="11">
         <v>43655.570870476193</v>
       </c>
-    </row>
-    <row r="122" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A122" s="88" t="s">
+      <c r="V121" s="11">
+        <v>115.35</v>
+      </c>
+    </row>
+    <row r="122" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A122" s="95" t="s">
         <v>970</v>
       </c>
       <c r="B122" s="88">
@@ -14215,18 +14821,24 @@
       <c r="Q122" s="92">
         <v>4.63</v>
       </c>
-      <c r="R122" s="11">
+      <c r="R122" s="92">
         <v>44.84</v>
       </c>
-      <c r="S122" s="11">
+      <c r="S122">
+        <v>71.7</v>
+      </c>
+      <c r="T122" s="11">
         <v>19565.044000000002</v>
       </c>
-      <c r="T122" s="11">
+      <c r="U122" s="11">
         <v>43524.348633499998</v>
       </c>
-    </row>
-    <row r="123" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A123" s="89" t="s">
+      <c r="V122" s="11">
+        <v>113.37</v>
+      </c>
+    </row>
+    <row r="123" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A123" s="96" t="s">
         <v>971</v>
       </c>
       <c r="B123" s="89">
@@ -14277,18 +14889,24 @@
       <c r="Q123" s="92">
         <v>4.45</v>
       </c>
-      <c r="R123" s="11">
+      <c r="R123" s="92">
         <v>45.31</v>
       </c>
-      <c r="S123" s="11">
+      <c r="S123">
+        <v>64.7</v>
+      </c>
+      <c r="T123" s="11">
         <v>19547.280999999999</v>
       </c>
-      <c r="T123" s="11">
+      <c r="U123" s="11">
         <v>44209.309622631583</v>
       </c>
-    </row>
-    <row r="124" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A124" s="88" t="s">
+      <c r="V123" s="11">
+        <v>111.7</v>
+      </c>
+    </row>
+    <row r="124" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A124" s="95" t="s">
         <v>972</v>
       </c>
       <c r="B124" s="88">
@@ -14339,18 +14957,24 @@
       <c r="Q124" s="92">
         <v>4.28</v>
       </c>
-      <c r="R124" s="11">
+      <c r="R124" s="92">
         <v>43.45</v>
       </c>
-      <c r="S124" s="11">
+      <c r="S124">
+        <v>57</v>
+      </c>
+      <c r="T124" s="11">
         <v>17828.026000000002</v>
       </c>
-      <c r="T124" s="11">
+      <c r="U124" s="11">
         <v>42092.12872047619</v>
       </c>
-    </row>
-    <row r="125" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A125" s="89" t="s">
+      <c r="V124" s="11">
+        <v>112.13</v>
+      </c>
+    </row>
+    <row r="125" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A125" s="96" t="s">
         <v>973</v>
       </c>
       <c r="B125" s="89">
@@ -14401,18 +15025,24 @@
       <c r="Q125" s="92">
         <v>4.28</v>
       </c>
-      <c r="R125" s="11">
+      <c r="R125" s="92">
         <v>42.38</v>
       </c>
-      <c r="S125" s="11">
+      <c r="S125">
+        <v>52.2</v>
+      </c>
+      <c r="T125" s="11">
         <v>16678.46</v>
       </c>
-      <c r="T125" s="11">
+      <c r="U125" s="11">
         <v>39876.327753809521</v>
       </c>
-    </row>
-    <row r="126" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A126" s="88" t="s">
+      <c r="V125" s="11">
+        <v>115.28</v>
+      </c>
+    </row>
+    <row r="126" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A126" s="95" t="s">
         <v>974</v>
       </c>
       <c r="B126" s="88">
@@ -14463,18 +15093,24 @@
       <c r="Q126" s="92">
         <v>4.42</v>
       </c>
-      <c r="R126" s="11">
+      <c r="R126" s="92">
         <v>42.45</v>
       </c>
-      <c r="S126" s="11">
+      <c r="S126">
+        <v>52.2</v>
+      </c>
+      <c r="T126" s="11">
         <v>18642.367999999999</v>
       </c>
-      <c r="T126" s="11">
+      <c r="U126" s="11">
         <v>41864.245349999997</v>
       </c>
-    </row>
-    <row r="127" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A127" s="89" t="s">
+      <c r="V126" s="11">
+        <v>119.22</v>
+      </c>
+    </row>
+    <row r="127" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A127" s="96" t="s">
         <v>975</v>
       </c>
       <c r="B127" s="89">
@@ -14525,18 +15161,24 @@
       <c r="Q127" s="92">
         <v>4.38</v>
       </c>
-      <c r="R127" s="11">
+      <c r="R127" s="92">
         <v>43.85</v>
       </c>
-      <c r="S127" s="11">
+      <c r="S127">
+        <v>60.7</v>
+      </c>
+      <c r="T127" s="11">
         <v>19673.300999999999</v>
       </c>
-      <c r="T127" s="11">
+      <c r="U127" s="11">
         <v>42752.938085000002</v>
       </c>
-    </row>
-    <row r="128" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A128" s="88" t="s">
+      <c r="V127" s="11">
+        <v>120.41</v>
+      </c>
+    </row>
+    <row r="128" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A128" s="95" t="s">
         <v>976</v>
       </c>
       <c r="B128" s="88">
@@ -14587,18 +15229,24 @@
       <c r="Q128" s="92">
         <v>4.3899999999999997</v>
       </c>
-      <c r="R128" s="11">
+      <c r="R128" s="92">
         <v>47.22</v>
       </c>
-      <c r="S128" s="11">
+      <c r="S128">
+        <v>61.7</v>
+      </c>
+      <c r="T128" s="11">
         <v>20784.895</v>
       </c>
-      <c r="T128" s="11">
+      <c r="U128" s="11">
         <v>44499.741300909089</v>
       </c>
-    </row>
-    <row r="129" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A129" s="89" t="s">
+      <c r="V128" s="11">
+        <v>121.31</v>
+      </c>
+    </row>
+    <row r="129" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A129" s="96" t="s">
         <v>977</v>
       </c>
       <c r="B129" s="89">
@@ -14649,18 +15297,24 @@
       <c r="Q129" s="92">
         <v>4.26</v>
       </c>
-      <c r="R129" s="11">
+      <c r="R129" s="92">
         <v>37.08</v>
       </c>
-      <c r="S129" s="11">
+      <c r="S129">
+        <v>58.2</v>
+      </c>
+      <c r="T129" s="11">
         <v>21383.587</v>
       </c>
-      <c r="T129" s="11">
+      <c r="U129" s="11">
         <v>44764.850632857153</v>
       </c>
-    </row>
-    <row r="130" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A130" s="88" t="s">
+      <c r="V129" s="11">
+        <v>122.4</v>
+      </c>
+    </row>
+    <row r="130" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A130" s="95" t="s">
         <v>978</v>
       </c>
       <c r="B130" s="88">
@@ -14711,18 +15365,24 @@
       <c r="Q130" s="92">
         <v>4.12</v>
       </c>
-      <c r="R130" s="11">
+      <c r="R130" s="92">
         <v>40.630000000000003</v>
       </c>
-      <c r="S130" s="11">
+      <c r="S130">
+        <v>55.1</v>
+      </c>
+      <c r="T130" s="11">
         <v>22188.588</v>
       </c>
-      <c r="T130" s="11">
+      <c r="U130" s="11">
         <v>45908.102306666668</v>
       </c>
-    </row>
-    <row r="131" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A131" s="89" t="s">
+      <c r="V130" s="11">
+        <v>122.44</v>
+      </c>
+    </row>
+    <row r="131" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A131" s="96" t="s">
         <v>979</v>
       </c>
       <c r="B131" s="89">
@@ -14773,18 +15433,24 @@
       <c r="Q131" s="92">
         <v>4.0599999999999996</v>
       </c>
-      <c r="R131" s="11">
+      <c r="R131" s="92">
         <v>40.33</v>
       </c>
-      <c r="S131" s="11">
+      <c r="S131">
+        <v>53.6</v>
+      </c>
+      <c r="T131" s="11">
         <v>23003.126</v>
       </c>
-      <c r="T131" s="11">
+      <c r="U131" s="11">
         <v>46709.672214782608</v>
       </c>
-    </row>
-    <row r="132" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A132" s="88" t="s">
+      <c r="V131" s="11">
+        <v>124.81</v>
+      </c>
+    </row>
+    <row r="132" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A132" s="95" t="s">
         <v>980</v>
       </c>
       <c r="B132" s="88">
@@ -14835,18 +15501,24 @@
       <c r="Q132" s="92">
         <v>4.09</v>
       </c>
-      <c r="R132" s="11">
+      <c r="R132" s="92">
         <v>39.92</v>
       </c>
-      <c r="S132" s="11">
+      <c r="S132">
+        <v>51</v>
+      </c>
+      <c r="T132" s="11">
         <v>23023.623</v>
       </c>
-      <c r="T132" s="11">
+      <c r="U132" s="11">
         <v>47016.374177894737</v>
       </c>
-    </row>
-    <row r="133" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A133" s="89" t="s">
+      <c r="V132" s="11">
+        <v>129.56</v>
+      </c>
+    </row>
+    <row r="133" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A133" s="96" t="s">
         <v>981</v>
       </c>
       <c r="B133" s="89">
@@ -14897,18 +15569,24 @@
       <c r="Q133" s="92">
         <v>4.1399999999999997</v>
       </c>
-      <c r="R133" s="11">
+      <c r="R133" s="92">
         <v>48.31</v>
       </c>
-      <c r="S133" s="11">
+      <c r="S133">
+        <v>52.9</v>
+      </c>
+      <c r="T133" s="11">
         <v>23377.327000000001</v>
       </c>
-      <c r="T133" s="11">
+      <c r="U133" s="11">
         <v>48118.866655454549</v>
       </c>
-    </row>
-    <row r="134" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A134" s="88" t="s">
+      <c r="V133" s="11">
+        <v>132.19</v>
+      </c>
+    </row>
+    <row r="134" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A134" s="95" t="s">
         <v>982</v>
       </c>
       <c r="B134" s="88">
@@ -14959,18 +15637,24 @@
       <c r="Q134" s="92">
         <v>4.21</v>
       </c>
-      <c r="R134" s="11">
+      <c r="R134" s="92">
         <v>47.59</v>
       </c>
-      <c r="S134" s="11">
+      <c r="S134">
+        <v>56.4</v>
+      </c>
+      <c r="T134" s="11">
         <v>23520.722000000002</v>
       </c>
-      <c r="T134" s="11">
+      <c r="U134" s="11">
         <v>49138.273634500001</v>
       </c>
-    </row>
-    <row r="135" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A135" s="89" t="s">
+      <c r="V134" s="11">
+        <v>134.99</v>
+      </c>
+    </row>
+    <row r="135" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A135" s="96" t="s">
         <v>983</v>
       </c>
       <c r="B135" s="89">
@@ -15021,18 +15705,24 @@
       <c r="Q135" s="92">
         <v>4.13</v>
       </c>
-      <c r="R135" s="11">
+      <c r="R135" s="92">
         <v>43.89</v>
       </c>
-      <c r="S135" s="11">
+      <c r="S135">
+        <v>56.6</v>
+      </c>
+      <c r="T135" s="11">
         <v>22892.922999999999</v>
       </c>
-      <c r="T135" s="11">
+      <c r="U135" s="11">
         <v>49511.972041052628</v>
       </c>
-    </row>
-    <row r="136" spans="1:20" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A136" s="88" t="s">
+      <c r="V135" s="11">
+        <v>138.80000000000001</v>
+      </c>
+    </row>
+    <row r="136" spans="1:22" s="11" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A136" s="95" t="s">
         <v>984</v>
       </c>
       <c r="B136" s="88">
@@ -15083,53 +15773,61 @@
       <c r="Q136" s="92">
         <v>4.25</v>
       </c>
-      <c r="R136" s="11">
+      <c r="R136" s="92">
         <v>40.83</v>
       </c>
-      <c r="S136" s="11">
+      <c r="S136">
+        <v>53.3</v>
+      </c>
+      <c r="T136" s="11">
         <v>22130.038</v>
       </c>
-      <c r="T136" s="11">
+      <c r="U136" s="11">
         <v>46859.672230909091</v>
       </c>
-    </row>
-    <row r="137" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="V136" s="11">
+        <v>137.88</v>
+      </c>
+    </row>
+    <row r="137" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A137" s="90"/>
       <c r="B137" s="90"/>
       <c r="P137" s="94">
         <v>3.8</v>
       </c>
       <c r="Q137" s="92"/>
-    </row>
-    <row r="138" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="R137" s="92"/>
+    </row>
+    <row r="138" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A138" s="90"/>
       <c r="B138" s="90"/>
       <c r="P138" s="94">
         <v>4</v>
       </c>
       <c r="Q138" s="92"/>
-    </row>
-    <row r="139" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="R138" s="92"/>
+    </row>
+    <row r="139" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A139" s="90"/>
       <c r="B139" s="90"/>
     </row>
-    <row r="140" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A140" s="90"/>
       <c r="B140" s="90"/>
     </row>
-    <row r="141" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A141" s="90"/>
       <c r="B141" s="90"/>
     </row>
-    <row r="142" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A142" s="90"/>
       <c r="B142" s="90"/>
     </row>
-    <row r="143" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A143" s="90"/>
       <c r="B143" s="90"/>
     </row>
-    <row r="144" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:22" x14ac:dyDescent="0.35">
       <c r="A144" s="90"/>
       <c r="B144" s="90"/>
     </row>
@@ -15312,7 +16010,7 @@
       <c r="N6" s="43"/>
       <c r="O6" s="43"/>
       <c r="P6" s="44"/>
-      <c r="Q6" s="97" t="s">
+      <c r="Q6" s="99" t="s">
         <v>131</v>
       </c>
     </row>
@@ -15321,10 +16019,10 @@
       <c r="B7" s="78"/>
       <c r="C7" s="38"/>
       <c r="D7" s="39"/>
-      <c r="E7" s="98" t="s">
+      <c r="E7" s="100" t="s">
         <v>1010</v>
       </c>
-      <c r="F7" s="99"/>
+      <c r="F7" s="101"/>
       <c r="G7" s="27"/>
       <c r="H7" s="27"/>
       <c r="I7" s="27"/>
@@ -15335,11 +16033,11 @@
       <c r="N7" s="31" t="s">
         <v>993</v>
       </c>
-      <c r="O7" s="100" t="s">
+      <c r="O7" s="102" t="s">
         <v>64</v>
       </c>
-      <c r="P7" s="101"/>
-      <c r="Q7" s="97"/>
+      <c r="P7" s="103"/>
+      <c r="Q7" s="99"/>
     </row>
     <row r="8" spans="1:80" ht="16.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="17"/>
@@ -15363,7 +16061,7 @@
       <c r="M8" s="26"/>
       <c r="N8" s="32"/>
       <c r="O8" s="34"/>
-      <c r="P8" s="95" t="s">
+      <c r="P8" s="97" t="s">
         <v>137</v>
       </c>
       <c r="Q8" s="39"/>
@@ -15404,7 +16102,7 @@
         <v>111</v>
       </c>
       <c r="O9" s="35"/>
-      <c r="P9" s="96"/>
+      <c r="P9" s="98"/>
       <c r="Q9" s="45" t="s">
         <v>111</v>
       </c>
@@ -76604,39 +77302,39 @@
         <v>102</v>
       </c>
       <c r="B77" s="60"/>
-      <c r="C77" s="102" t="s">
+      <c r="C77" s="104" t="s">
         <v>101</v>
       </c>
-      <c r="D77" s="102"/>
-      <c r="E77" s="102"/>
-      <c r="F77" s="102"/>
-      <c r="G77" s="102"/>
-      <c r="H77" s="102"/>
-      <c r="I77" s="102"/>
-      <c r="J77" s="102"/>
-      <c r="K77" s="102"/>
-      <c r="L77" s="102"/>
-      <c r="M77" s="102"/>
-      <c r="N77" s="102"/>
-      <c r="O77" s="102"/>
+      <c r="D77" s="104"/>
+      <c r="E77" s="104"/>
+      <c r="F77" s="104"/>
+      <c r="G77" s="104"/>
+      <c r="H77" s="104"/>
+      <c r="I77" s="104"/>
+      <c r="J77" s="104"/>
+      <c r="K77" s="104"/>
+      <c r="L77" s="104"/>
+      <c r="M77" s="104"/>
+      <c r="N77" s="104"/>
+      <c r="O77" s="104"/>
       <c r="P77" s="60"/>
     </row>
     <row r="78" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A78" s="60"/>
       <c r="B78" s="60"/>
-      <c r="C78" s="102"/>
-      <c r="D78" s="102"/>
-      <c r="E78" s="102"/>
-      <c r="F78" s="102"/>
-      <c r="G78" s="102"/>
-      <c r="H78" s="102"/>
-      <c r="I78" s="102"/>
-      <c r="J78" s="102"/>
-      <c r="K78" s="102"/>
-      <c r="L78" s="102"/>
-      <c r="M78" s="102"/>
-      <c r="N78" s="102"/>
-      <c r="O78" s="102"/>
+      <c r="C78" s="104"/>
+      <c r="D78" s="104"/>
+      <c r="E78" s="104"/>
+      <c r="F78" s="104"/>
+      <c r="G78" s="104"/>
+      <c r="H78" s="104"/>
+      <c r="I78" s="104"/>
+      <c r="J78" s="104"/>
+      <c r="K78" s="104"/>
+      <c r="L78" s="104"/>
+      <c r="M78" s="104"/>
+      <c r="N78" s="104"/>
+      <c r="O78" s="104"/>
       <c r="P78" s="60"/>
     </row>
     <row r="79" spans="1:16" x14ac:dyDescent="0.35">
@@ -76644,75 +77342,75 @@
         <v>124</v>
       </c>
       <c r="B79" s="60"/>
-      <c r="C79" s="102" t="s">
+      <c r="C79" s="104" t="s">
         <v>103</v>
       </c>
-      <c r="D79" s="102"/>
-      <c r="E79" s="102"/>
-      <c r="F79" s="102"/>
-      <c r="G79" s="102"/>
-      <c r="H79" s="102"/>
-      <c r="I79" s="102"/>
-      <c r="J79" s="102"/>
-      <c r="K79" s="102"/>
-      <c r="L79" s="102"/>
-      <c r="M79" s="102"/>
-      <c r="N79" s="102"/>
-      <c r="O79" s="102"/>
+      <c r="D79" s="104"/>
+      <c r="E79" s="104"/>
+      <c r="F79" s="104"/>
+      <c r="G79" s="104"/>
+      <c r="H79" s="104"/>
+      <c r="I79" s="104"/>
+      <c r="J79" s="104"/>
+      <c r="K79" s="104"/>
+      <c r="L79" s="104"/>
+      <c r="M79" s="104"/>
+      <c r="N79" s="104"/>
+      <c r="O79" s="104"/>
       <c r="P79" s="60"/>
     </row>
     <row r="80" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A80" s="60"/>
       <c r="B80" s="60"/>
-      <c r="C80" s="102"/>
-      <c r="D80" s="102"/>
-      <c r="E80" s="102"/>
-      <c r="F80" s="102"/>
-      <c r="G80" s="102"/>
-      <c r="H80" s="102"/>
-      <c r="I80" s="102"/>
-      <c r="J80" s="102"/>
-      <c r="K80" s="102"/>
-      <c r="L80" s="102"/>
-      <c r="M80" s="102"/>
-      <c r="N80" s="102"/>
-      <c r="O80" s="102"/>
+      <c r="C80" s="104"/>
+      <c r="D80" s="104"/>
+      <c r="E80" s="104"/>
+      <c r="F80" s="104"/>
+      <c r="G80" s="104"/>
+      <c r="H80" s="104"/>
+      <c r="I80" s="104"/>
+      <c r="J80" s="104"/>
+      <c r="K80" s="104"/>
+      <c r="L80" s="104"/>
+      <c r="M80" s="104"/>
+      <c r="N80" s="104"/>
+      <c r="O80" s="104"/>
       <c r="P80" s="60"/>
     </row>
     <row r="81" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A81" s="60"/>
       <c r="B81" s="60"/>
-      <c r="C81" s="102"/>
-      <c r="D81" s="102"/>
-      <c r="E81" s="102"/>
-      <c r="F81" s="102"/>
-      <c r="G81" s="102"/>
-      <c r="H81" s="102"/>
-      <c r="I81" s="102"/>
-      <c r="J81" s="102"/>
-      <c r="K81" s="102"/>
-      <c r="L81" s="102"/>
-      <c r="M81" s="102"/>
-      <c r="N81" s="102"/>
-      <c r="O81" s="102"/>
+      <c r="C81" s="104"/>
+      <c r="D81" s="104"/>
+      <c r="E81" s="104"/>
+      <c r="F81" s="104"/>
+      <c r="G81" s="104"/>
+      <c r="H81" s="104"/>
+      <c r="I81" s="104"/>
+      <c r="J81" s="104"/>
+      <c r="K81" s="104"/>
+      <c r="L81" s="104"/>
+      <c r="M81" s="104"/>
+      <c r="N81" s="104"/>
+      <c r="O81" s="104"/>
       <c r="P81" s="60"/>
     </row>
     <row r="82" spans="1:16" x14ac:dyDescent="0.35">
       <c r="A82" s="60"/>
       <c r="B82" s="60"/>
-      <c r="C82" s="102"/>
-      <c r="D82" s="102"/>
-      <c r="E82" s="102"/>
-      <c r="F82" s="102"/>
-      <c r="G82" s="102"/>
-      <c r="H82" s="102"/>
-      <c r="I82" s="102"/>
-      <c r="J82" s="102"/>
-      <c r="K82" s="102"/>
-      <c r="L82" s="102"/>
-      <c r="M82" s="102"/>
-      <c r="N82" s="102"/>
-      <c r="O82" s="102"/>
+      <c r="C82" s="104"/>
+      <c r="D82" s="104"/>
+      <c r="E82" s="104"/>
+      <c r="F82" s="104"/>
+      <c r="G82" s="104"/>
+      <c r="H82" s="104"/>
+      <c r="I82" s="104"/>
+      <c r="J82" s="104"/>
+      <c r="K82" s="104"/>
+      <c r="L82" s="104"/>
+      <c r="M82" s="104"/>
+      <c r="N82" s="104"/>
+      <c r="O82" s="104"/>
       <c r="P82" s="60"/>
     </row>
     <row r="83" spans="1:16" x14ac:dyDescent="0.35">

</xml_diff>